<commit_message>
Add customised cold email for every lead and make it part of each batch
- batches/emails_data.py: subject and body for all 60 leads, with opt-out sign-off
- Workbook: email address, subject and body in Leads; email sent, follow-up due and sent in Tracker
- batches/cold-emails.md and batch 02 doc now include the emails
- .claude/skills/gliped-lead-batch: batch workflow with cold email rules, so future batches ship with emails
- Playbook: cold email section

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCxqvUeG6omvZWYGiRrK1m
</commit_message>
<xml_diff>
--- a/Gliped_Outreach_Tracker.xlsx
+++ b/Gliped_Outreach_Tracker.xlsx
@@ -15,8 +15,8 @@
     <sheet name="Lists" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Leads'!$A$1:$W$61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$Y$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Leads'!$A$1:$Z$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$AC$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -700,78 +700,90 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Days since last touch</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Days since the latest date you've entered in that row.</t>
+          <t>Paste the verified work email in Leads (Email address). Tracker shows it and counts Email sent + 5 days for the email follow-up. Send LinkedIn first; email is the second channel for leads who don't accept or reply.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>Days since last touch</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Days since the latest date you've entered in that row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>Yellow cells</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>The only cells you need to edit. Grey or white cells are formulas or reference data.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr"/>
-      <c r="B17" s="2" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Example row (format only)</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>G999 | Status: DM sent | Warm-up started 2026-09-26 | Connection sent 2026-10-01 | Accepted 2026-10-02 | First DM sent 2026-10-02 | FU1 due fills in as 2026-10-06 | Next action: send FU1 teardown offer</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
-      <c r="B19" s="2" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Scoring</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Trigger in last 90 days (max 30) + profile gap (max 20) + fit (10) + active in last 30 days (10). Intent signals were not visible, so add +30 by hand when someone views your profile or engages with Gliped. Tier: 60+ Priority, 40 to 59 Warm, under 40 Nurture.</t>
-        </is>
-      </c>
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Profile confirmed = No</t>
+          <t>Scoring</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>The LinkedIn link is a people search. Open it, match company and role, then paste the real profile URL into Leads and set Profile confirmed to Yes.</t>
+          <t>Trigger in last 90 days (max 30) + profile gap (max 20) + fit (10) + active in last 30 days (10). Intent signals were not visible, so add +30 by hand when someone views your profile or engages with Gliped. Tier: 60+ Priority, 40 to 59 Warm, under 40 Nurture.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
+          <t>Profile confirmed = No</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>The LinkedIn link is a people search. Open it, match company and role, then paste the real profile URL into Leads and set Profile confirmed to Yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>Activity data</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Posting timelines come from publicly indexed LinkedIn posts, dated from each post's activity ID. The index only catches some posts, so 'last indexed own post' means at least that recent.</t>
         </is>
@@ -788,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W61"/>
+  <dimension ref="A1:Z61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -814,6 +826,9 @@
     <col width="45" customWidth="1" min="21" max="21"/>
     <col width="40" customWidth="1" min="22" max="22"/>
     <col width="36" customWidth="1" min="23" max="23"/>
+    <col width="26" customWidth="1" min="24" max="24"/>
+    <col width="26" customWidth="1" min="25" max="25"/>
+    <col width="60" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -932,6 +947,21 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="X1" s="6" t="inlineStr">
+        <is>
+          <t>Email address</t>
+        </is>
+      </c>
+      <c r="Y1" s="6" t="inlineStr">
+        <is>
+          <t>Email subject</t>
+        </is>
+      </c>
+      <c r="Z1" s="6" t="inlineStr">
+        <is>
+          <t>Email body</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="96" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -1042,6 +1072,24 @@
           <t>India. Warm, respectful tone. Expect a CoS or comms lead in the decision.</t>
         </is>
       </c>
+      <c r="X2" s="9" t="inlineStr"/>
+      <c r="Y2" s="7" t="inlineStr">
+        <is>
+          <t>Nua after the Series C</t>
+        </is>
+      </c>
+      <c r="Z2" s="7" t="inlineStr">
+        <is>
+          <t>Hi Ravi,
+Congrats on the $50M Series C.
+Nua's story gets told at big moments, like the Zero to Scale episode, then it goes quiet. In women's wellness, the founder's voice is a trust asset between campaigns too.
+We run LinkedIn for founders: strategy, writing and posting, built around your voice.
+Worth a 15-minute call next week to see what that could look like for you?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="96" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
@@ -1151,6 +1199,24 @@
           <t>India, early stage and price-conscious. Lead with a starter plan and mention the pilot option early.</t>
         </is>
       </c>
+      <c r="X3" s="9" t="inlineStr"/>
+      <c r="Y3" s="7" t="inlineStr">
+        <is>
+          <t>Firi's founder story</t>
+        </is>
+      </c>
+      <c r="Z3" s="7" t="inlineStr">
+        <is>
+          <t>Hi Karishma,
+Nine-minute beauty delivery and a seed round in the same quarter. Strong start.
+In beauty, people buy from people. Right now Firi's story lives in press coverage, not on your LinkedIn, and that's where hires, partners and your next investors will look.
+We build founder brands on LinkedIn, from positioning to weekly posts.
+Open to a quick call to map out your first 90 days?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="96" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -1261,6 +1327,24 @@
           <t>UK. Plain and understated. "Might be useful" over "huge opportunity".</t>
         </is>
       </c>
+      <c r="X4" s="9" t="inlineStr"/>
+      <c r="Y4" s="7" t="inlineStr">
+        <is>
+          <t>Ryft's European push</t>
+        </is>
+      </c>
+      <c r="Z4" s="7" t="inlineStr">
+        <is>
+          <t>Hi Sadra,
+Congrats on the EUR 23M and the move into Europe.
+Buyers in new markets will look you up before they take a call. Your last post was in April 2025, and your FCA licence post shows your audience responds when you do post.
+We help founders turn that into a steady weekly presence without eating their week.
+Worth 15 minutes to talk through a Europe-facing plan?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="96" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -1371,6 +1455,24 @@
           <t>Canada. Polite and practical. If you email, CASL applies: it must be relevant to her role and include an unsubscribe. CASL applies to email</t>
         </is>
       </c>
+      <c r="X5" s="9" t="inlineStr"/>
+      <c r="Y5" s="7" t="inlineStr">
+        <is>
+          <t>askpolly's US launch</t>
+        </is>
+      </c>
+      <c r="Z5" s="7" t="inlineStr">
+        <is>
+          <t>Hi Erin,
+Congrats on the seed and the US go-to-market push.
+askpolly turns social conversations into insight. That kind of data does very well on LinkedIn, and right now none of it goes out under your name to the US buyers you want to reach.
+We build founder brands on LinkedIn, one insight post a week to start.
+Open to a 15-minute call to sketch it out?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="96" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -1481,6 +1583,24 @@
           <t>US, based in SF, with an India connection. Be direct but warm.</t>
         </is>
       </c>
+      <c r="X6" s="9" t="inlineStr"/>
+      <c r="Y6" s="7" t="inlineStr">
+        <is>
+          <t>Cradlewise, new markets</t>
+        </is>
+      </c>
+      <c r="Z6" s="7" t="inlineStr">
+        <is>
+          <t>Hi Radhika,
+Congrats on the Series A and the international push.
+You've built great press around Cradlewise, but your own LinkedIn has been quiet since mid-2023. New retail partners and parents will look you up first.
+We run LinkedIn for founders: positioning, writing and a steady posting rhythm in your voice.
+Would a 15-minute call next week be useful?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="96" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -1591,6 +1711,24 @@
           <t>SF and Bengaluru. Use a US-direct tone and offer IST or PT slots.</t>
         </is>
       </c>
+      <c r="X7" s="9" t="inlineStr"/>
+      <c r="Y7" s="7" t="inlineStr">
+        <is>
+          <t>Flam and US CMOs</t>
+        </is>
+      </c>
+      <c r="Z7" s="7" t="inlineStr">
+        <is>
+          <t>Hi Shourya,
+Congrats on the $40M Series B.
+Flam sells interactive content to CMOs, yet your feed is mostly launch announcements. CMOs follow people with a point of view, and yours is the story behind Flam.
+We help founders build that voice on LinkedIn, from strategy to weekly posts.
+Open to 15 minutes to talk through a US-facing plan?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="96" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1701,6 +1839,24 @@
           <t>same company as lead 19. Message Jagnoor first. Don't contact Shashank in the same week. If Jagnoor replies, the pitch can grow into a leadership pair (founder plus CEO). Contact before Shashank ND</t>
         </is>
       </c>
+      <c r="X8" s="9" t="inlineStr"/>
+      <c r="Y8" s="7" t="inlineStr">
+        <is>
+          <t>Your first 100 days</t>
+        </is>
+      </c>
+      <c r="Z8" s="7" t="inlineStr">
+        <is>
+          <t>Hi Jagnoor,
+Congrats on stepping in as Practo's CEO.
+The first months in the seat are when the market decides what a CEO stands for. Your posts get real engagement (56 comments on #growprofitably), but they come about once a quarter.
+We help CXOs turn that into a steady, credible weekly presence with little time from them.
+Worth a 15-minute call to map your first 100 days on LinkedIn?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="96" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
@@ -1811,6 +1967,24 @@
           <t>confirm where she's based before sending (India or US) and set the tone to match. Confirm location</t>
         </is>
       </c>
+      <c r="X9" s="9" t="inlineStr"/>
+      <c r="Y9" s="7" t="inlineStr">
+        <is>
+          <t>VerifAIX, trust first</t>
+        </is>
+      </c>
+      <c r="Z9" s="7" t="inlineStr">
+        <is>
+          <t>Hi Madhulima,
+Congrats on the $5M seed.
+In chip verification a handful of senior engineers decide who they trust. Right now VerifAIX shows up at events like the RISC-V Summit, but not much on LinkedIn between them.
+We build technical founder brands on LinkedIn, aimed at the few people who matter.
+Open to a quick call to see if it fits?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="96" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -1921,6 +2095,24 @@
           <t>UK, and North of England. Keep it low-key and skip the hype words.</t>
         </is>
       </c>
+      <c r="X10" s="9" t="inlineStr"/>
+      <c r="Y10" s="7" t="inlineStr">
+        <is>
+          <t>Back to posting?</t>
+        </is>
+      </c>
+      <c r="Z10" s="7" t="inlineStr">
+        <is>
+          <t>Hi Ben,
+Congrats on the Series A.
+You used to post regularly on LinkedIn, then it went quiet around 2024. The round was announced by others, not you.
+Enterprise security buyers respond to founders they recognise. We help founders get back to a steady rhythm without writing every post themselves.
+Worth 15 minutes next week to talk it through?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="96" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
@@ -2031,6 +2223,24 @@
           <t>UK. Direct and specific. He'll spot generic copy immediately. Check for in-house marketing</t>
         </is>
       </c>
+      <c r="X11" s="9" t="inlineStr"/>
+      <c r="Y11" s="7" t="inlineStr">
+        <is>
+          <t>The CloudNC story, restarted</t>
+        </is>
+      </c>
+      <c r="Z11" s="7" t="inlineStr">
+        <is>
+          <t>Hi Theo,
+Congrats on the new round.
+In 2023 you told the CloudNC story yourself on LinkedIn. Since early 2024 the storytelling has moved to the company page.
+Machinists and manufacturers follow you, not the logo. We help founders restart and keep that rhythm, with you in control of the voice.
+Open to a 15-minute call to see what a restart could look like?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="96" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -2141,6 +2351,24 @@
           <t>Canada, Toronto. Polite and practical.</t>
         </is>
       </c>
+      <c r="X12" s="9" t="inlineStr"/>
+      <c r="Y12" s="7" t="inlineStr">
+        <is>
+          <t>Fisent's story, your voice</t>
+        </is>
+      </c>
+      <c r="Z12" s="7" t="inlineStr">
+        <is>
+          <t>Hi Adrian,
+Congrats on the raise.
+Other people keep telling Fisent's story in interviews, but your own LinkedIn has been quiet since mid-2025. Outcomes-as-a-service is a strong idea to own in public.
+We turn founders' thinking into a steady LinkedIn presence for enterprise buyers.
+Worth a 15-minute call to see how?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="96" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
@@ -2251,6 +2479,24 @@
           <t>Canada, Toronto, with a US and YC audience. Short and direct.</t>
         </is>
       </c>
+      <c r="X13" s="9" t="inlineStr"/>
+      <c r="Y13" s="7" t="inlineStr">
+        <is>
+          <t>Hiring after the Series A</t>
+        </is>
+      </c>
+      <c r="Z13" s="7" t="inlineStr">
+        <is>
+          <t>Hi Raghav,
+Congrats on the $20M Series A.
+Your LinkedIn is mostly job posts right now. Strong engineers pick founders whose thinking they've already seen.
+We help technical founders write about the problem they're solving, so hiring and fleet buyers come to them.
+Open to 15 minutes to talk it through?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="96" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -2361,6 +2607,24 @@
           <t>Canada, Alberta. Respectful. He likely has advisers, so expect a gatekeeper. Former Alberta minister</t>
         </is>
       </c>
+      <c r="X14" s="9" t="inlineStr"/>
+      <c r="Y14" s="7" t="inlineStr">
+        <is>
+          <t>From minister to founder</t>
+        </is>
+      </c>
+      <c r="Z14" s="7" t="inlineStr">
+        <is>
+          <t>Hi Doug,
+Congrats on Ultimarii's Series A.
+People know you from your years in government. Fewer know you yet as the founder speeding up infrastructure approvals with AI, and your LinkedIn still reads like the old role.
+We help founders reposition on LinkedIn with a steady voice aimed at energy and infrastructure leaders.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="96" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -2471,6 +2735,24 @@
           <t>Quebec. Offer French. Polite and practical. Active last 30 days; offer French</t>
         </is>
       </c>
+      <c r="X15" s="9" t="inlineStr"/>
+      <c r="Y15" s="7" t="inlineStr">
+        <is>
+          <t>Scopia's next chapter</t>
+        </is>
+      </c>
+      <c r="Z15" s="7" t="inlineStr">
+        <is>
+          <t>Hi Gabriel,
+Congrats on closing the pre-seed.
+In medtech, surgeons and partners check the founder before the product. Right now you post at milestones only.
+We build founder brands on LinkedIn, in English, French or both, aimed at clinicians and partners.
+Open to a quick call to see what that could look like for Scopia?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="96" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -2581,6 +2863,24 @@
           <t>confirm his location (assumed US). Direct and numbers-first. Confirm location</t>
         </is>
       </c>
+      <c r="X16" s="9" t="inlineStr"/>
+      <c r="Y16" s="7" t="inlineStr">
+        <is>
+          <t>Bootstrapped to Series A</t>
+        </is>
+      </c>
+      <c r="Z16" s="7" t="inlineStr">
+        <is>
+          <t>Hi David,
+Congrats on the Series A. Bootstrapping to that point in payments is rare.
+That's a story banks and platforms want to hear, but your LinkedIn has been quiet since 2023.
+We help founders turn their thinking into a steady LinkedIn presence, aimed at the partners they need.
+Worth 15 minutes to talk it through?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="96" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
@@ -2691,6 +2991,24 @@
           <t>UK. Pre-seed budget, so offer a lighter plan or pilot. Pre-seed budget</t>
         </is>
       </c>
+      <c r="X17" s="9" t="inlineStr"/>
+      <c r="Y17" s="7" t="inlineStr">
+        <is>
+          <t>Weekly, not quarterly</t>
+        </is>
+      </c>
+      <c r="Z17" s="7" t="inlineStr">
+        <is>
+          <t>Hi Leo,
+Congrats on the pre-seed.
+You already write about partnerships on LinkedIn, and your buyers live there. The gap is rhythm: a post every few months instead of every week.
+We help founders keep a weekly cadence in their own voice without it eating their week.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="96" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -2801,6 +3119,24 @@
           <t>UK. Precise and low-hype. Expect security-minded scepticism.</t>
         </is>
       </c>
+      <c r="X18" s="9" t="inlineStr"/>
+      <c r="Y18" s="7" t="inlineStr">
+        <is>
+          <t>AI governance, out loud</t>
+        </is>
+      </c>
+      <c r="Z18" s="7" t="inlineStr">
+        <is>
+          <t>Hi Alex,
+Congrats on the round.
+You have a clear point of view on AI governance, and CISOs and GCs need to hear it more than twice a year.
+We help founders turn that point of view into a steady LinkedIn presence that builds the category with them in it.
+Worth a 15-minute call next week?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="96" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
@@ -2911,6 +3247,24 @@
           <t>US East. Direct.</t>
         </is>
       </c>
+      <c r="X19" s="9" t="inlineStr"/>
+      <c r="Y19" s="7" t="inlineStr">
+        <is>
+          <t>Explaining Helogen</t>
+        </is>
+      </c>
+      <c r="Z19" s="7" t="inlineStr">
+        <is>
+          <t>Hi Shishir,
+Congrats on the seed.
+Space biomanufacturing needs a lot of explaining to investors, talent and early customers. "The next industrial revolution isn't on earth" is a good frame, and it deserves a regular slot.
+We help frontier founders build an explainer-led presence on LinkedIn.
+Open to a quick call to see how?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="96" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -3017,6 +3371,24 @@
           <t>only after lead 7 has been contacted and at least a week has passed. The likely route is through his comms or CoS. India, senior. Very respectful and short. Wait 1 week after Jagnoor</t>
         </is>
       </c>
+      <c r="X20" s="9" t="inlineStr"/>
+      <c r="Y20" s="7" t="inlineStr">
+        <is>
+          <t>The chairman's voice</t>
+        </is>
+      </c>
+      <c r="Z20" s="7" t="inlineStr">
+        <is>
+          <t>Hi Shashank,
+Congratulations on the new role at Practo.
+Moving from CEO to Executive Chairman changes what people expect to hear from you: capital, AI and the long-term bets, not operations.
+We help senior leaders shape that narrative on LinkedIn, with a light touch on their time.
+Would a short call be useful, with you or whoever runs your comms?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="96" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
@@ -3127,6 +3499,24 @@
           <t>US West. Numbers-first. He'll judge Gliped on its own profile, so make sure it's current. Pitch time and reach not starting</t>
         </is>
       </c>
+      <c r="X21" s="9" t="inlineStr"/>
+      <c r="Y21" s="7" t="inlineStr">
+        <is>
+          <t>Your weekly hours back</t>
+        </is>
+      </c>
+      <c r="Z21" s="7" t="inlineStr">
+        <is>
+          <t>Hi Ilan,
+Congrats on the Series A.
+You're one of the few founders who posts consistently. That usually costs hours a week that a CEO of a fast-growing company doesn't have.
+We keep founders' voice and rhythm while taking the writing and repurposing off their plate.
+Worth 15 minutes to see what you'd get back?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="96" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -3245,6 +3635,24 @@
           <t>Co-founders Ujjwal Sukheja and Saran S. also post. Pitch Aniket first.</t>
         </is>
       </c>
+      <c r="X22" s="9" t="inlineStr"/>
+      <c r="Y22" s="7" t="inlineStr">
+        <is>
+          <t>Swish's founder story</t>
+        </is>
+      </c>
+      <c r="Z22" s="7" t="inlineStr">
+        <is>
+          <t>Hi Aniket,
+Congrats on the $24M round.
+Quick commerce is crowded, and Swish's story mostly shows up at raises and hiring posts. The founder who explains why 10-minute fresh food works wins the best hires and the press in between.
+We build founder brands on LinkedIn, from positioning to weekly posts.
+Open to a 15-minute call next week?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="96" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
@@ -3363,6 +3771,24 @@
           <t>Deep tech, government and defence buyers. Keep it formal.</t>
         </is>
       </c>
+      <c r="X23" s="9" t="inlineStr"/>
+      <c r="Y23" s="7" t="inlineStr">
+        <is>
+          <t>Quantum-safe, explained</t>
+        </is>
+      </c>
+      <c r="Z23" s="7" t="inlineStr">
+        <is>
+          <t>Hi Sunil,
+Congrats on the Rs 200 Cr Series A1.
+Your LinkedIn announces QNu's milestones well. What most CISOs and government buyers still need is the why: why quantum-safe, why now.
+We help deep-tech founders build that voice on LinkedIn, steadily and credibly.
+Worth a 15-minute call to see how it could work for you?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="96" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
@@ -3481,6 +3907,24 @@
           <t>Check whether he already posts on YouTube or X. If so, pitch repurposing onto LinkedIn.</t>
         </is>
       </c>
+      <c r="X24" s="9" t="inlineStr"/>
+      <c r="Y24" s="7" t="inlineStr">
+        <is>
+          <t>Your credentials, visible</t>
+        </is>
+      </c>
+      <c r="Z24" s="7" t="inlineStr">
+        <is>
+          <t>Hi Prashant,
+Congrats on the pre-Series A.
+You carry more technical-analysis credentials than most people posting about markets, yet they barely show on LinkedIn. Retail traders follow people, not platforms.
+We turn founders' expertise into a steady LinkedIn presence that pulls users to the product.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="96" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
@@ -3599,6 +4043,24 @@
           <t>Co-founder brother Nikhil Gupta. Pitch AB first.</t>
         </is>
       </c>
+      <c r="X25" s="9" t="inlineStr"/>
+      <c r="Y25" s="7" t="inlineStr">
+        <is>
+          <t>Pizza Bakery, next cities</t>
+        </is>
+      </c>
+      <c r="Z25" s="7" t="inlineStr">
+        <is>
+          <t>Hi AB,
+Congrats on the Rs 532 Cr round from Artal.
+You built The Pizza Bakery without growth capital. That's a founder story F&amp;B operators, landlords and new-city hires will follow, and it hasn't been on your LinkedIn since 2023.
+We build founder brands on LinkedIn around stories like that.
+Worth 15 minutes to talk it through?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="96" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
@@ -3713,6 +4175,24 @@
           <t>Confirm profile before sending.</t>
         </is>
       </c>
+      <c r="X26" s="9" t="inlineStr"/>
+      <c r="Y26" s="7" t="inlineStr">
+        <is>
+          <t>Profitable from month one</t>
+        </is>
+      </c>
+      <c r="Z26" s="7" t="inlineStr">
+        <is>
+          <t>Hi Karan,
+Congrats on the Uber-led round.
+A second-time founder, profitable from month one, backed twice by Uber. Very few people in mobility can tell that story, and right now you're not telling it on LinkedIn.
+We build founder brands on LinkedIn, from positioning to weekly posts.
+Open to a 15-minute call next week?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="96" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
@@ -3823,6 +4303,24 @@
           <t>Confirm profile before sending.</t>
         </is>
       </c>
+      <c r="X27" s="9" t="inlineStr"/>
+      <c r="Y27" s="7" t="inlineStr">
+        <is>
+          <t>Cooling as a category</t>
+        </is>
+      </c>
+      <c r="Z27" s="7" t="inlineStr">
+        <is>
+          <t>Hi Abhishek,
+Congrats on the pre-Series A.
+Cooling-as-a-service is a new category, and businesses buying it want to trust the operator behind it. Right now Circolife's page does the talking.
+We help founders build their own voice on LinkedIn around the category they're creating.
+Worth a quick call to see if it fits?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="96" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
@@ -3937,6 +4435,24 @@
           <t>Confirm profile. Co-founder Nishanth Jois.</t>
         </is>
       </c>
+      <c r="X28" s="9" t="inlineStr"/>
+      <c r="Y28" s="7" t="inlineStr">
+        <is>
+          <t>UniqYou's launch voice</t>
+        </is>
+      </c>
+      <c r="Z28" s="7" t="inlineStr">
+        <is>
+          <t>Hi Sneha,
+Congrats on the seed, and on backers like the Myntra founders.
+In fashion, people buy into the founder's taste first. A founder-led LinkedIn at launch often costs less than paid acquisition and brings hires with it.
+We build founder brands on LinkedIn from day one.
+Open to 15 minutes to plan your first 90 days?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="96" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
@@ -4051,6 +4567,24 @@
           <t>Confirm profile. Co-founder Sandeep Upadhyay. Medical advertising rules apply to content.</t>
         </is>
       </c>
+      <c r="X29" s="9" t="inlineStr"/>
+      <c r="Y29" s="7" t="inlineStr">
+        <is>
+          <t>TRUE ARTIS, trust first</t>
+        </is>
+      </c>
+      <c r="Z29" s="7" t="inlineStr">
+        <is>
+          <t>Hi Ankit,
+Congrats on the seed.
+In aesthetic surgery, patients check who's behind the clinic before they book. A founder who talks openly about safety and standards sets TRUE ARTIS apart.
+We build founder brands on LinkedIn, carefully and within medical advertising norms.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="96" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
@@ -4165,6 +4699,24 @@
           <t>Confirm profile. This is debt financing, not equity, so avoid calling it a round.</t>
         </is>
       </c>
+      <c r="X30" s="9" t="inlineStr"/>
+      <c r="Y30" s="7" t="inlineStr">
+        <is>
+          <t>Greenwave and ESG buyers</t>
+        </is>
+      </c>
+      <c r="Z30" s="7" t="inlineStr">
+        <is>
+          <t>Hi Devang,
+Congrats on the OeEB financing.
+The brand sustainability leads you'll want as offtake partners are on LinkedIn. A founder voice on closed-loop PET recycling gives them a reason to call you first.
+We build founder brands on LinkedIn, aimed at the buyers that matter.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="96" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
@@ -4275,6 +4827,24 @@
           <t>Confirm profile. Pre-seed budget, so offer the pilot.</t>
         </is>
       </c>
+      <c r="X31" s="9" t="inlineStr"/>
+      <c r="Y31" s="7" t="inlineStr">
+        <is>
+          <t>24 prototypes is content</t>
+        </is>
+      </c>
+      <c r="Z31" s="7" t="inlineStr">
+        <is>
+          <t>Hi Avni,
+Congrats on the pre-seed.
+24 prototypes and 900 hours of wear testing to get a heel that doesn't hurt. That build story is content most D2C founders would kill for.
+We help founders turn stories like that into a steady LinkedIn presence, sized for an early-stage budget.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="96" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
@@ -4393,6 +4963,24 @@
           <t>Likely has comms support. Ask who owns his LinkedIn.</t>
         </is>
       </c>
+      <c r="X32" s="9" t="inlineStr"/>
+      <c r="Y32" s="7" t="inlineStr">
+        <is>
+          <t>Scan.com's US chapter</t>
+        </is>
+      </c>
+      <c r="Z32" s="7" t="inlineStr">
+        <is>
+          <t>Hi Charlie,
+Congrats on the Series C and the US push.
+Your posts land well when you post, but the last one I could find was March 2025. US health systems and partners are meeting you for the first time now.
+We help founders keep a steady, credible LinkedIn presence, working with your comms team.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="96" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
@@ -4511,6 +5099,24 @@
           <t>The 'resigns' post is an April Fools joke. He's still CEO.</t>
         </is>
       </c>
+      <c r="X33" s="9" t="inlineStr"/>
+      <c r="Y33" s="7" t="inlineStr">
+        <is>
+          <t>Rightcharge across Europe</t>
+        </is>
+      </c>
+      <c r="Z33" s="7" t="inlineStr">
+        <is>
+          <t>Hi Charlie,
+Congrats on the raise and the Visa partnership.
+You've got a real voice on LinkedIn, humour included. It just shows up a few times a year, and European fleet managers don't know you yet.
+We help founders keep a weekly rhythm in their own voice without it eating their week.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="96" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
@@ -4625,6 +5231,24 @@
         </is>
       </c>
       <c r="W34" s="7" t="inlineStr"/>
+      <c r="X34" s="9" t="inlineStr"/>
+      <c r="Y34" s="7" t="inlineStr">
+        <is>
+          <t>Making Ki 13 stick</t>
+        </is>
+      </c>
+      <c r="Z34" s="7" t="inlineStr">
+        <is>
+          <t>Hi Koji,
+Congrats on the seed and the new Ki 13 name.
+A rebrand only sticks when people hear the story behind it, and right now you post mainly at milestones.
+We help deep-tech founders build a steady LinkedIn presence that explains the science and the ambition.
+Worth 15 minutes to talk it through?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="96" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
@@ -4739,6 +5363,24 @@
         </is>
       </c>
       <c r="W35" s="7" t="inlineStr"/>
+      <c r="X35" s="9" t="inlineStr"/>
+      <c r="Y35" s="7" t="inlineStr">
+        <is>
+          <t>Your own AI visibility</t>
+        </is>
+      </c>
+      <c r="Z35" s="7" t="inlineStr">
+        <is>
+          <t>Hi Francisco,
+Congrats on the seed.
+Odd one for someone in AI visibility: LinkedIn posts are one of the sources AI models draw on, and right now the geoSurge company page does most of the talking.
+We build founder brands on LinkedIn, so the founder shows up too.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="96" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
@@ -4857,6 +5499,24 @@
           <t>Co-founder Dr Sam Tukra.</t>
         </is>
       </c>
+      <c r="X36" s="9" t="inlineStr"/>
+      <c r="Y36" s="7" t="inlineStr">
+        <is>
+          <t>Orbital, in your words</t>
+        </is>
+      </c>
+      <c r="Z36" s="7" t="inlineStr">
+        <is>
+          <t>Hi Callum,
+Congrats on the round with KBR and Databricks.
+Energy operators buy from people they trust, and a CEO voice on AI in refining is rare. Right now Orbital's story lives on the company page.
+We help founders build a steady LinkedIn presence aimed at operators.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="96" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
@@ -4975,6 +5635,24 @@
           <t>Co-founder Max Clarke. Big brand, so expect a comms team.</t>
         </is>
       </c>
+      <c r="X37" s="9" t="inlineStr"/>
+      <c r="Y37" s="7" t="inlineStr">
+        <is>
+          <t>Healf, week by week</t>
+        </is>
+      </c>
+      <c r="Z37" s="7" t="inlineStr">
+        <is>
+          <t>Hi Lestat,
+Congrats on the round and the Germany launch.
+Your AI adoption piece got people talking, but it's one of only a few posts. With international growth and press momentum, a steady rhythm compounds.
+We help founders keep a weekly LinkedIn presence in their own voice, alongside their comms team.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="96" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
@@ -5093,6 +5771,24 @@
           <t>Low fit for ghostwriting. Only pitch strategy.</t>
         </is>
       </c>
+      <c r="X38" s="9" t="inlineStr"/>
+      <c r="Y38" s="7" t="inlineStr">
+        <is>
+          <t>Distribution, not writing</t>
+        </is>
+      </c>
+      <c r="Z38" s="7" t="inlineStr">
+        <is>
+          <t>Hi Jon,
+Congrats on the Marker launch.
+You write your own posts and should. For most writer-founders the harder part is distribution: cadence, formats and reaching buyers, not only other writers.
+That's the part we can help with at Gliped, with you still doing the writing.
+Worth a 15-minute chat?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="96" customHeight="1">
       <c r="A39" s="7" t="inlineStr">
@@ -5211,6 +5907,24 @@
           <t>Confirm who's CEO (Stephen or Joshua Hampson).</t>
         </is>
       </c>
+      <c r="X39" s="9" t="inlineStr"/>
+      <c r="Y39" s="7" t="inlineStr">
+        <is>
+          <t>Keeping it weekly</t>
+        </is>
+      </c>
+      <c r="Z39" s="7" t="inlineStr">
+        <is>
+          <t>Hi Stephen,
+Congrats on the seed.
+You've started posting customer stories on LinkedIn, which is the right instinct for reaching pharma commercial teams. The hard part is keeping it going every week.
+We help founders do exactly that, in their own voice.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="96" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
@@ -5321,6 +6035,24 @@
           <t>Confirm profile and whether he's the founder.</t>
         </is>
       </c>
+      <c r="X40" s="9" t="inlineStr"/>
+      <c r="Y40" s="7" t="inlineStr">
+        <is>
+          <t>Tickets for Good's story</t>
+        </is>
+      </c>
+      <c r="Z40" s="7" t="inlineStr">
+        <is>
+          <t>Hi Steve,
+Congrats on the new funding.
+Getting surplus tickets to key workers is the kind of story people share, and venues and promoters respond to the person behind it.
+We build founder brands on LinkedIn around stories like yours.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="96" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
@@ -5434,6 +6166,24 @@
           <t>Confirm profile and base (UK or US).</t>
         </is>
       </c>
+      <c r="X41" s="9" t="inlineStr"/>
+      <c r="Y41" s="7" t="inlineStr">
+        <is>
+          <t>Expanse on both sides</t>
+        </is>
+      </c>
+      <c r="Z41" s="7" t="inlineStr">
+        <is>
+          <t>Hi Ismaeel,
+Congrats on the raise.
+AI infrastructure is noisy, and with teams in the UK and US you need buyers on both sides to recognise you. A clear founder point of view on LinkedIn does that.
+We build founder brands on LinkedIn, from positioning to weekly posts.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="96" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
@@ -5548,6 +6298,24 @@
           <t>Confirm profile.</t>
         </is>
       </c>
+      <c r="X42" s="9" t="inlineStr"/>
+      <c r="Y42" s="7" t="inlineStr">
+        <is>
+          <t>Mundo's founder voice</t>
+        </is>
+      </c>
+      <c r="Z42" s="7" t="inlineStr">
+        <is>
+          <t>Hi Jason,
+Congrats on the Series A.
+Most of Mundo's story online comes from press and your co-founders. Model teams and top researchers want to hear from the CEO too.
+We build founder brands on LinkedIn for technical founders, aimed at buyers and hires.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="96" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
@@ -5666,6 +6434,24 @@
           <t>Writer himself, so pitch strategy over ghostwriting.</t>
         </is>
       </c>
+      <c r="X43" s="9" t="inlineStr"/>
+      <c r="Y43" s="7" t="inlineStr">
+        <is>
+          <t>Onix and your voice</t>
+        </is>
+      </c>
+      <c r="Z43" s="7" t="inlineStr">
+        <is>
+          <t>Hi David,
+Congrats on the pre-seed.
+Onix is built on experts owning their voice. Yours shows up on LinkedIn every few months.
+You can clearly write, so this isn't about ghostwriting. We help founders with cadence, formats and distribution.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="96" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
@@ -5784,6 +6570,24 @@
           <t>Likely has an in-house comms team. Pitch executive content support.</t>
         </is>
       </c>
+      <c r="X44" s="9" t="inlineStr"/>
+      <c r="Y44" s="7" t="inlineStr">
+        <is>
+          <t>Fullscript's CEO voice</t>
+        </is>
+      </c>
+      <c r="Z44" s="7" t="inlineStr">
+        <is>
+          <t>Hi Kyle,
+Congrats on the L Catterton and Altas investment.
+Your LinkedIn is mostly Fullscript updates. Practitioners and partners would follow a stronger CEO point of view on where integrative health is going.
+We support executive LinkedIn presence alongside in-house comms teams.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="96" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
@@ -5902,6 +6706,24 @@
           <t>Montreal. Offer French.</t>
         </is>
       </c>
+      <c r="X45" s="9" t="inlineStr"/>
+      <c r="Y45" s="7" t="inlineStr">
+        <is>
+          <t>Terra Mobility, restarted</t>
+        </is>
+      </c>
+      <c r="Z45" s="7" t="inlineStr">
+        <is>
+          <t>Hi LP,
+Congrats on the financing and the Terra Mobility launch.
+Your LatAm and Africa posts drew 60+ comments, then your LinkedIn went quiet in 2024. A new parent company is the moment to restart.
+We help founders get back to a steady rhythm without writing every post themselves.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="96" customHeight="1">
       <c r="A46" s="7" t="inlineStr">
@@ -6020,6 +6842,24 @@
           <t>Confirm the funding date before sending. Write in French.</t>
         </is>
       </c>
+      <c r="X46" s="9" t="inlineStr"/>
+      <c r="Y46" s="7" t="inlineStr">
+        <is>
+          <t>Micrologic et le cloud souverain</t>
+        </is>
+      </c>
+      <c r="Z46" s="7" t="inlineStr">
+        <is>
+          <t>Bonjour Stéphane,
+Félicitations pour le financement.
+Le cloud souverain est un sujet d'actualité, et vous publiiez régulièrement là-dessus jusqu'en 2024. Une voix de PDG, en français et en anglais, positionne Micrologic auprès des acheteurs publics.
+Chez Gliped, nous bâtissons la présence LinkedIn des dirigeants.
+Un appel de 15 minutes la semaine prochaine?
+Prabal
+Gliped | Personal branding LinkedIn pour dirigeants
+Pas pertinent? Répondez « non » et je ne vous relancerai pas.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="96" customHeight="1">
       <c r="A47" s="7" t="inlineStr">
@@ -6138,6 +6978,24 @@
           <t>High profile. Low odds, high value.</t>
         </is>
       </c>
+      <c r="X47" s="9" t="inlineStr"/>
+      <c r="Y47" s="7" t="inlineStr">
+        <is>
+          <t>Veeda, from NVIDIA</t>
+        </is>
+      </c>
+      <c r="Z47" s="7" t="inlineStr">
+        <is>
+          <t>Hi Sanja,
+Congrats on launching Veeda.
+Your LinkedIn has been NVIDIA research. Veeda is a new story, and the researchers you want to hire will look for it in your feed.
+We help technical founders build a founder narrative on LinkedIn without pulling them away from the work.
+Worth a short call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="96" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
@@ -6255,6 +7113,24 @@
           <t>Nurture. Trigger is older than 90 days. Revisit on the next trigger.</t>
         </is>
       </c>
+      <c r="X48" s="9" t="inlineStr"/>
+      <c r="Y48" s="7" t="inlineStr">
+        <is>
+          <t>NationGraph, steadily</t>
+        </is>
+      </c>
+      <c r="Z48" s="7" t="inlineStr">
+        <is>
+          <t>Hi Kimia,
+Your NationGraph launch post drew a lot of discussion. Since then you post a few times a year.
+Public-sector buyers take time to trust a vendor, and a steady founder voice shortens that.
+We help founders keep a regular LinkedIn rhythm in their own voice.
+Open to a quick call when timing suits?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="96" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
@@ -6369,6 +7245,24 @@
           <t>Confirm profile.</t>
         </is>
       </c>
+      <c r="X49" s="9" t="inlineStr"/>
+      <c r="Y49" s="7" t="inlineStr">
+        <is>
+          <t>Legio and campus leaders</t>
+        </is>
+      </c>
+      <c r="Z49" s="7" t="inlineStr">
+        <is>
+          <t>Hi Darren,
+Congrats on the seed.
+Campus safety leaders are a tight community, and they buy on trust. A founder voice on LinkedIn about safety operations sets Legio apart.
+We build founder brands on LinkedIn aimed at the buyers that matter.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="96" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
@@ -6483,6 +7377,24 @@
           <t>Confirm profile. Co-founder Mustafa Khan.</t>
         </is>
       </c>
+      <c r="X50" s="9" t="inlineStr"/>
+      <c r="Y50" s="7" t="inlineStr">
+        <is>
+          <t>Peripheral on LinkedIn</t>
+        </is>
+      </c>
+      <c r="Z50" s="7" t="inlineStr">
+        <is>
+          <t>Hi Kelvin,
+Congrats on the seed.
+Your product is very visual, which suits LinkedIn. Founder posts with product clips double as marketing to sports media buyers.
+We build founder brands on LinkedIn, from positioning to weekly posts.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="96" customHeight="1">
       <c r="A51" s="7" t="inlineStr">
@@ -6597,6 +7509,24 @@
           <t>Launch, not a funding round. Check whether there was a raise.</t>
         </is>
       </c>
+      <c r="X51" s="9" t="inlineStr"/>
+      <c r="Y51" s="7" t="inlineStr">
+        <is>
+          <t>MakeOS, founder-led</t>
+        </is>
+      </c>
+      <c r="Z51" s="7" t="inlineStr">
+        <is>
+          <t>Hi Sumit,
+Congrats on launching MakeOS.
+The launch is on the Makers page, but your own feed is quiet. Producers and agencies live on LinkedIn, and they follow people.
+We build founder brands on LinkedIn around launches like this one.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="96" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
@@ -6707,6 +7637,24 @@
         </is>
       </c>
       <c r="W52" s="7" t="inlineStr"/>
+      <c r="X52" s="9" t="inlineStr"/>
+      <c r="Y52" s="7" t="inlineStr">
+        <is>
+          <t>Light's founder voice</t>
+        </is>
+      </c>
+      <c r="Z52" s="7" t="inlineStr">
+        <is>
+          <t>Hi Baker,
+Congrats on the $46M Series A.
+Energy is a trust category, and your LinkedIn has been nearly silent. Brands deciding whether to launch their own electricity plan will look you up.
+We build founder brands on LinkedIn, from positioning to weekly posts.
+Open to a quick call next week?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="96" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
@@ -6821,6 +7769,24 @@
           <t>Active in the last 30 days.</t>
         </is>
       </c>
+      <c r="X53" s="9" t="inlineStr"/>
+      <c r="Y53" s="7" t="inlineStr">
+        <is>
+          <t>Your weekly hours back</t>
+        </is>
+      </c>
+      <c r="Z53" s="7" t="inlineStr">
+        <is>
+          <t>Hi Guy,
+Congrats on the Series A.
+You post more consistently than most founders. That usually costs hours a week, right when Blee is scaling.
+We keep founders' voice and rhythm while taking the writing and repurposing off their plate.
+Worth 15 minutes to see what you'd get back?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="96" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
@@ -6939,6 +7905,24 @@
           <t>Defence content has rules. Check export and ITAR boundaries.</t>
         </is>
       </c>
+      <c r="X54" s="9" t="inlineStr"/>
+      <c r="Y54" s="7" t="inlineStr">
+        <is>
+          <t>Aurelius, every week</t>
+        </is>
+      </c>
+      <c r="Z54" s="7" t="inlineStr">
+        <is>
+          <t>Hi Michael,
+Congrats on the $40M Series A.
+Your defence-tech posts get attention when they land, every month or two. Weekly would help both hiring and customers.
+We help founders keep that rhythm in their own voice, with care around what defence content can say.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="96" customHeight="1">
       <c r="A55" s="7" t="inlineStr">
@@ -7053,6 +8037,24 @@
         </is>
       </c>
       <c r="W55" s="7" t="inlineStr"/>
+      <c r="X55" s="9" t="inlineStr"/>
+      <c r="Y55" s="7" t="inlineStr">
+        <is>
+          <t>TerraFirma, weekly</t>
+        </is>
+      </c>
+      <c r="Z55" s="7" t="inlineStr">
+        <is>
+          <t>Hi Noah,
+Congrats on the Series A.
+You post with a clear point of view every couple of months. Weekly turns that into a category voice for construction.
+We help founders keep a weekly rhythm in their own voice without it eating their week.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="96" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
@@ -7167,6 +8169,24 @@
           <t>Co-founders Aryamika Bhatia Ondaatje and Sasivarnan K S.</t>
         </is>
       </c>
+      <c r="X56" s="9" t="inlineStr"/>
+      <c r="Y56" s="7" t="inlineStr">
+        <is>
+          <t>Aranya out of stealth</t>
+        </is>
+      </c>
+      <c r="Z56" s="7" t="inlineStr">
+        <is>
+          <t>Hi Christian,
+Congrats on the raise.
+Aranya's story is on the company page and your co-founder's feed. Infrastructure buyers want to hear from the CEO, and yours has been quiet since 2024.
+We build founder brands on LinkedIn for technical founders.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="96" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
@@ -7285,6 +8305,24 @@
           <t>Forbes 30 Under 30 with co-founder Vikhyat Chaudhry.</t>
         </is>
       </c>
+      <c r="X57" s="9" t="inlineStr"/>
+      <c r="Y57" s="7" t="inlineStr">
+        <is>
+          <t>Buzz and utility buyers</t>
+        </is>
+      </c>
+      <c r="Z57" s="7" t="inlineStr">
+        <is>
+          <t>Hi Kaitlyn,
+Congrats on the Series A.
+You post at big moments and do interviews well. Utilities are conservative buyers, and a steady CEO voice on grid reliability builds trust that press alone doesn't.
+We help founders turn interviews and milestones into a weekly LinkedIn rhythm.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="96" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
@@ -7399,6 +8437,24 @@
           <t>Co-founder CTO Antonin Parrot.</t>
         </is>
       </c>
+      <c r="X58" s="9" t="inlineStr"/>
+      <c r="Y58" s="7" t="inlineStr">
+        <is>
+          <t>River Markets, weekly</t>
+        </is>
+      </c>
+      <c r="Z58" s="7" t="inlineStr">
+        <is>
+          <t>Hi Oscar,
+Congrats on the seed.
+You've just started posting about prediction markets. The founder who shows up every week for institutions becomes the category voice.
+We help founders keep that rhythm while they deploy a new round.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="96" customHeight="1">
       <c r="A59" s="7" t="inlineStr">
@@ -7509,6 +8565,24 @@
           <t>Confirm profile.</t>
         </is>
       </c>
+      <c r="X59" s="9" t="inlineStr"/>
+      <c r="Y59" s="7" t="inlineStr">
+        <is>
+          <t>Foundational's story</t>
+        </is>
+      </c>
+      <c r="Z59" s="7" t="inlineStr">
+        <is>
+          <t>Hi Adel,
+Congrats on the $25M seed.
+American reshoring plus AI-native factories is a story people want to follow, and right now you're not telling it on LinkedIn.
+We build founder brands on LinkedIn, from positioning to weekly posts, including build-in-public.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="96" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
@@ -7623,6 +8697,24 @@
           <t>Confirm profile. Sensitive topic, so keep it measured.</t>
         </is>
       </c>
+      <c r="X60" s="9" t="inlineStr"/>
+      <c r="Y60" s="7" t="inlineStr">
+        <is>
+          <t>Blue Voice's why</t>
+        </is>
+      </c>
+      <c r="Z60" s="7" t="inlineStr">
+        <is>
+          <t>Hi David,
+Congrats on the raise.
+Why you left law school to build Blue Voice is a story police leaders and councils would read, and it builds the trust public-safety buyers need.
+We build founder brands on LinkedIn, carefully and in a measured tone.
+Open to a quick call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="96" customHeight="1">
       <c r="A61" s="7" t="inlineStr">
@@ -7737,9 +8829,27 @@
           <t>Confirm profile and who the CEO is. Co-founders Ben Finch and Ryan Winkler.</t>
         </is>
       </c>
+      <c r="X61" s="9" t="inlineStr"/>
+      <c r="Y61" s="7" t="inlineStr">
+        <is>
+          <t>Multiplier in New York</t>
+        </is>
+      </c>
+      <c r="Z61" s="7" t="inlineStr">
+        <is>
+          <t>Hi Ian,
+Congrats on the seed and the move to New York.
+Ryan has been the voice of the launch so far. At seed stage, the founder who posts gets the first hires' and first customers' attention.
+We build founder brands on LinkedIn, from positioning to weekly posts.
+Worth a 15-minute call?
+Prabal
+Gliped | LinkedIn personal branding for founders
+Not relevant? Reply "no" and I won't follow up.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W61"/>
+  <autoFilter ref="A1:Z61"/>
   <conditionalFormatting sqref="J2:J261">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"No"</formula>
@@ -7867,7 +8977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y61"/>
+  <dimension ref="A1:AC61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7895,6 +9005,10 @@
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="10" customWidth="1" min="24" max="24"/>
     <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="24" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -8021,6 +9135,26 @@
       <c r="Y1" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="Z1" s="6" t="inlineStr">
+        <is>
+          <t>Email address</t>
+        </is>
+      </c>
+      <c r="AA1" s="6" t="inlineStr">
+        <is>
+          <t>Email sent</t>
+        </is>
+      </c>
+      <c r="AB1" s="6" t="inlineStr">
+        <is>
+          <t>Email FU due</t>
+        </is>
+      </c>
+      <c r="AC1" s="6" t="inlineStr">
+        <is>
+          <t>Email FU sent</t>
         </is>
       </c>
     </row>
@@ -8081,10 +9215,20 @@
       <c r="V2" s="9" t="n"/>
       <c r="W2" s="13" t="n"/>
       <c r="X2" s="11">
-        <f>IF(MAX(I2:L2,N2,P2:S2)=0,"",TODAY()-MAX(I2:L2,N2,P2:S2))</f>
+        <f>IF(MAX(I2:L2,N2,P2:S2,AA2,AC2)=0,"",TODAY()-MAX(I2:L2,N2,P2:S2,AA2,AC2))</f>
         <v/>
       </c>
       <c r="Y2" s="9" t="n"/>
+      <c r="Z2" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A2,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A2,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA2" s="13" t="n"/>
+      <c r="AB2" s="14">
+        <f>IF(AA2="","",AA2+5)</f>
+        <v/>
+      </c>
+      <c r="AC2" s="13" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
@@ -8143,10 +9287,20 @@
       <c r="V3" s="9" t="n"/>
       <c r="W3" s="13" t="n"/>
       <c r="X3" s="11">
-        <f>IF(MAX(I3:L3,N3,P3:S3)=0,"",TODAY()-MAX(I3:L3,N3,P3:S3))</f>
+        <f>IF(MAX(I3:L3,N3,P3:S3,AA3,AC3)=0,"",TODAY()-MAX(I3:L3,N3,P3:S3,AA3,AC3))</f>
         <v/>
       </c>
       <c r="Y3" s="9" t="n"/>
+      <c r="Z3" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A3,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A3,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA3" s="13" t="n"/>
+      <c r="AB3" s="14">
+        <f>IF(AA3="","",AA3+5)</f>
+        <v/>
+      </c>
+      <c r="AC3" s="13" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -8205,10 +9359,20 @@
       <c r="V4" s="9" t="n"/>
       <c r="W4" s="13" t="n"/>
       <c r="X4" s="11">
-        <f>IF(MAX(I4:L4,N4,P4:S4)=0,"",TODAY()-MAX(I4:L4,N4,P4:S4))</f>
+        <f>IF(MAX(I4:L4,N4,P4:S4,AA4,AC4)=0,"",TODAY()-MAX(I4:L4,N4,P4:S4,AA4,AC4))</f>
         <v/>
       </c>
       <c r="Y4" s="9" t="n"/>
+      <c r="Z4" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A4,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A4,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA4" s="13" t="n"/>
+      <c r="AB4" s="14">
+        <f>IF(AA4="","",AA4+5)</f>
+        <v/>
+      </c>
+      <c r="AC4" s="13" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -8267,10 +9431,20 @@
       <c r="V5" s="9" t="n"/>
       <c r="W5" s="13" t="n"/>
       <c r="X5" s="11">
-        <f>IF(MAX(I5:L5,N5,P5:S5)=0,"",TODAY()-MAX(I5:L5,N5,P5:S5))</f>
+        <f>IF(MAX(I5:L5,N5,P5:S5,AA5,AC5)=0,"",TODAY()-MAX(I5:L5,N5,P5:S5,AA5,AC5))</f>
         <v/>
       </c>
       <c r="Y5" s="9" t="n"/>
+      <c r="Z5" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A5,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A5,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA5" s="13" t="n"/>
+      <c r="AB5" s="14">
+        <f>IF(AA5="","",AA5+5)</f>
+        <v/>
+      </c>
+      <c r="AC5" s="13" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -8329,10 +9503,20 @@
       <c r="V6" s="9" t="n"/>
       <c r="W6" s="13" t="n"/>
       <c r="X6" s="11">
-        <f>IF(MAX(I6:L6,N6,P6:S6)=0,"",TODAY()-MAX(I6:L6,N6,P6:S6))</f>
+        <f>IF(MAX(I6:L6,N6,P6:S6,AA6,AC6)=0,"",TODAY()-MAX(I6:L6,N6,P6:S6,AA6,AC6))</f>
         <v/>
       </c>
       <c r="Y6" s="9" t="n"/>
+      <c r="Z6" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A6,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A6,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA6" s="13" t="n"/>
+      <c r="AB6" s="14">
+        <f>IF(AA6="","",AA6+5)</f>
+        <v/>
+      </c>
+      <c r="AC6" s="13" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -8391,10 +9575,20 @@
       <c r="V7" s="9" t="n"/>
       <c r="W7" s="13" t="n"/>
       <c r="X7" s="11">
-        <f>IF(MAX(I7:L7,N7,P7:S7)=0,"",TODAY()-MAX(I7:L7,N7,P7:S7))</f>
+        <f>IF(MAX(I7:L7,N7,P7:S7,AA7,AC7)=0,"",TODAY()-MAX(I7:L7,N7,P7:S7,AA7,AC7))</f>
         <v/>
       </c>
       <c r="Y7" s="9" t="n"/>
+      <c r="Z7" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A7,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A7,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA7" s="13" t="n"/>
+      <c r="AB7" s="14">
+        <f>IF(AA7="","",AA7+5)</f>
+        <v/>
+      </c>
+      <c r="AC7" s="13" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -8453,10 +9647,20 @@
       <c r="V8" s="9" t="n"/>
       <c r="W8" s="13" t="n"/>
       <c r="X8" s="11">
-        <f>IF(MAX(I8:L8,N8,P8:S8)=0,"",TODAY()-MAX(I8:L8,N8,P8:S8))</f>
+        <f>IF(MAX(I8:L8,N8,P8:S8,AA8,AC8)=0,"",TODAY()-MAX(I8:L8,N8,P8:S8,AA8,AC8))</f>
         <v/>
       </c>
       <c r="Y8" s="9" t="n"/>
+      <c r="Z8" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A8,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A8,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA8" s="13" t="n"/>
+      <c r="AB8" s="14">
+        <f>IF(AA8="","",AA8+5)</f>
+        <v/>
+      </c>
+      <c r="AC8" s="13" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -8515,10 +9719,20 @@
       <c r="V9" s="9" t="n"/>
       <c r="W9" s="13" t="n"/>
       <c r="X9" s="11">
-        <f>IF(MAX(I9:L9,N9,P9:S9)=0,"",TODAY()-MAX(I9:L9,N9,P9:S9))</f>
+        <f>IF(MAX(I9:L9,N9,P9:S9,AA9,AC9)=0,"",TODAY()-MAX(I9:L9,N9,P9:S9,AA9,AC9))</f>
         <v/>
       </c>
       <c r="Y9" s="9" t="n"/>
+      <c r="Z9" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A9,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A9,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA9" s="13" t="n"/>
+      <c r="AB9" s="14">
+        <f>IF(AA9="","",AA9+5)</f>
+        <v/>
+      </c>
+      <c r="AC9" s="13" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -8577,10 +9791,20 @@
       <c r="V10" s="9" t="n"/>
       <c r="W10" s="13" t="n"/>
       <c r="X10" s="11">
-        <f>IF(MAX(I10:L10,N10,P10:S10)=0,"",TODAY()-MAX(I10:L10,N10,P10:S10))</f>
+        <f>IF(MAX(I10:L10,N10,P10:S10,AA10,AC10)=0,"",TODAY()-MAX(I10:L10,N10,P10:S10,AA10,AC10))</f>
         <v/>
       </c>
       <c r="Y10" s="9" t="n"/>
+      <c r="Z10" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A10,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A10,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA10" s="13" t="n"/>
+      <c r="AB10" s="14">
+        <f>IF(AA10="","",AA10+5)</f>
+        <v/>
+      </c>
+      <c r="AC10" s="13" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -8639,10 +9863,20 @@
       <c r="V11" s="9" t="n"/>
       <c r="W11" s="13" t="n"/>
       <c r="X11" s="11">
-        <f>IF(MAX(I11:L11,N11,P11:S11)=0,"",TODAY()-MAX(I11:L11,N11,P11:S11))</f>
+        <f>IF(MAX(I11:L11,N11,P11:S11,AA11,AC11)=0,"",TODAY()-MAX(I11:L11,N11,P11:S11,AA11,AC11))</f>
         <v/>
       </c>
       <c r="Y11" s="9" t="n"/>
+      <c r="Z11" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A11,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A11,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA11" s="13" t="n"/>
+      <c r="AB11" s="14">
+        <f>IF(AA11="","",AA11+5)</f>
+        <v/>
+      </c>
+      <c r="AC11" s="13" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -8701,10 +9935,20 @@
       <c r="V12" s="9" t="n"/>
       <c r="W12" s="13" t="n"/>
       <c r="X12" s="11">
-        <f>IF(MAX(I12:L12,N12,P12:S12)=0,"",TODAY()-MAX(I12:L12,N12,P12:S12))</f>
+        <f>IF(MAX(I12:L12,N12,P12:S12,AA12,AC12)=0,"",TODAY()-MAX(I12:L12,N12,P12:S12,AA12,AC12))</f>
         <v/>
       </c>
       <c r="Y12" s="9" t="n"/>
+      <c r="Z12" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A12,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A12,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA12" s="13" t="n"/>
+      <c r="AB12" s="14">
+        <f>IF(AA12="","",AA12+5)</f>
+        <v/>
+      </c>
+      <c r="AC12" s="13" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -8763,10 +10007,20 @@
       <c r="V13" s="9" t="n"/>
       <c r="W13" s="13" t="n"/>
       <c r="X13" s="11">
-        <f>IF(MAX(I13:L13,N13,P13:S13)=0,"",TODAY()-MAX(I13:L13,N13,P13:S13))</f>
+        <f>IF(MAX(I13:L13,N13,P13:S13,AA13,AC13)=0,"",TODAY()-MAX(I13:L13,N13,P13:S13,AA13,AC13))</f>
         <v/>
       </c>
       <c r="Y13" s="9" t="n"/>
+      <c r="Z13" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A13,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A13,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA13" s="13" t="n"/>
+      <c r="AB13" s="14">
+        <f>IF(AA13="","",AA13+5)</f>
+        <v/>
+      </c>
+      <c r="AC13" s="13" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -8825,10 +10079,20 @@
       <c r="V14" s="9" t="n"/>
       <c r="W14" s="13" t="n"/>
       <c r="X14" s="11">
-        <f>IF(MAX(I14:L14,N14,P14:S14)=0,"",TODAY()-MAX(I14:L14,N14,P14:S14))</f>
+        <f>IF(MAX(I14:L14,N14,P14:S14,AA14,AC14)=0,"",TODAY()-MAX(I14:L14,N14,P14:S14,AA14,AC14))</f>
         <v/>
       </c>
       <c r="Y14" s="9" t="n"/>
+      <c r="Z14" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A14,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A14,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA14" s="13" t="n"/>
+      <c r="AB14" s="14">
+        <f>IF(AA14="","",AA14+5)</f>
+        <v/>
+      </c>
+      <c r="AC14" s="13" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -8887,10 +10151,20 @@
       <c r="V15" s="9" t="n"/>
       <c r="W15" s="13" t="n"/>
       <c r="X15" s="11">
-        <f>IF(MAX(I15:L15,N15,P15:S15)=0,"",TODAY()-MAX(I15:L15,N15,P15:S15))</f>
+        <f>IF(MAX(I15:L15,N15,P15:S15,AA15,AC15)=0,"",TODAY()-MAX(I15:L15,N15,P15:S15,AA15,AC15))</f>
         <v/>
       </c>
       <c r="Y15" s="9" t="n"/>
+      <c r="Z15" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A15,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A15,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA15" s="13" t="n"/>
+      <c r="AB15" s="14">
+        <f>IF(AA15="","",AA15+5)</f>
+        <v/>
+      </c>
+      <c r="AC15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
@@ -8949,10 +10223,20 @@
       <c r="V16" s="9" t="n"/>
       <c r="W16" s="13" t="n"/>
       <c r="X16" s="11">
-        <f>IF(MAX(I16:L16,N16,P16:S16)=0,"",TODAY()-MAX(I16:L16,N16,P16:S16))</f>
+        <f>IF(MAX(I16:L16,N16,P16:S16,AA16,AC16)=0,"",TODAY()-MAX(I16:L16,N16,P16:S16,AA16,AC16))</f>
         <v/>
       </c>
       <c r="Y16" s="9" t="n"/>
+      <c r="Z16" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A16,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A16,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA16" s="13" t="n"/>
+      <c r="AB16" s="14">
+        <f>IF(AA16="","",AA16+5)</f>
+        <v/>
+      </c>
+      <c r="AC16" s="13" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -9011,10 +10295,20 @@
       <c r="V17" s="9" t="n"/>
       <c r="W17" s="13" t="n"/>
       <c r="X17" s="11">
-        <f>IF(MAX(I17:L17,N17,P17:S17)=0,"",TODAY()-MAX(I17:L17,N17,P17:S17))</f>
+        <f>IF(MAX(I17:L17,N17,P17:S17,AA17,AC17)=0,"",TODAY()-MAX(I17:L17,N17,P17:S17,AA17,AC17))</f>
         <v/>
       </c>
       <c r="Y17" s="9" t="n"/>
+      <c r="Z17" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A17,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A17,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA17" s="13" t="n"/>
+      <c r="AB17" s="14">
+        <f>IF(AA17="","",AA17+5)</f>
+        <v/>
+      </c>
+      <c r="AC17" s="13" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
@@ -9073,10 +10367,20 @@
       <c r="V18" s="9" t="n"/>
       <c r="W18" s="13" t="n"/>
       <c r="X18" s="11">
-        <f>IF(MAX(I18:L18,N18,P18:S18)=0,"",TODAY()-MAX(I18:L18,N18,P18:S18))</f>
+        <f>IF(MAX(I18:L18,N18,P18:S18,AA18,AC18)=0,"",TODAY()-MAX(I18:L18,N18,P18:S18,AA18,AC18))</f>
         <v/>
       </c>
       <c r="Y18" s="9" t="n"/>
+      <c r="Z18" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A18,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A18,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA18" s="13" t="n"/>
+      <c r="AB18" s="14">
+        <f>IF(AA18="","",AA18+5)</f>
+        <v/>
+      </c>
+      <c r="AC18" s="13" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -9135,10 +10439,20 @@
       <c r="V19" s="9" t="n"/>
       <c r="W19" s="13" t="n"/>
       <c r="X19" s="11">
-        <f>IF(MAX(I19:L19,N19,P19:S19)=0,"",TODAY()-MAX(I19:L19,N19,P19:S19))</f>
+        <f>IF(MAX(I19:L19,N19,P19:S19,AA19,AC19)=0,"",TODAY()-MAX(I19:L19,N19,P19:S19,AA19,AC19))</f>
         <v/>
       </c>
       <c r="Y19" s="9" t="n"/>
+      <c r="Z19" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A19,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A19,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA19" s="13" t="n"/>
+      <c r="AB19" s="14">
+        <f>IF(AA19="","",AA19+5)</f>
+        <v/>
+      </c>
+      <c r="AC19" s="13" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
@@ -9197,10 +10511,20 @@
       <c r="V20" s="9" t="n"/>
       <c r="W20" s="13" t="n"/>
       <c r="X20" s="11">
-        <f>IF(MAX(I20:L20,N20,P20:S20)=0,"",TODAY()-MAX(I20:L20,N20,P20:S20))</f>
+        <f>IF(MAX(I20:L20,N20,P20:S20,AA20,AC20)=0,"",TODAY()-MAX(I20:L20,N20,P20:S20,AA20,AC20))</f>
         <v/>
       </c>
       <c r="Y20" s="9" t="n"/>
+      <c r="Z20" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A20,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A20,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA20" s="13" t="n"/>
+      <c r="AB20" s="14">
+        <f>IF(AA20="","",AA20+5)</f>
+        <v/>
+      </c>
+      <c r="AC20" s="13" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
@@ -9259,10 +10583,20 @@
       <c r="V21" s="9" t="n"/>
       <c r="W21" s="13" t="n"/>
       <c r="X21" s="11">
-        <f>IF(MAX(I21:L21,N21,P21:S21)=0,"",TODAY()-MAX(I21:L21,N21,P21:S21))</f>
+        <f>IF(MAX(I21:L21,N21,P21:S21,AA21,AC21)=0,"",TODAY()-MAX(I21:L21,N21,P21:S21,AA21,AC21))</f>
         <v/>
       </c>
       <c r="Y21" s="9" t="n"/>
+      <c r="Z21" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A21,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A21,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA21" s="13" t="n"/>
+      <c r="AB21" s="14">
+        <f>IF(AA21="","",AA21+5)</f>
+        <v/>
+      </c>
+      <c r="AC21" s="13" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
@@ -9321,10 +10655,20 @@
       <c r="V22" s="9" t="n"/>
       <c r="W22" s="13" t="n"/>
       <c r="X22" s="11">
-        <f>IF(MAX(I22:L22,N22,P22:S22)=0,"",TODAY()-MAX(I22:L22,N22,P22:S22))</f>
+        <f>IF(MAX(I22:L22,N22,P22:S22,AA22,AC22)=0,"",TODAY()-MAX(I22:L22,N22,P22:S22,AA22,AC22))</f>
         <v/>
       </c>
       <c r="Y22" s="9" t="n"/>
+      <c r="Z22" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A22,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A22,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA22" s="13" t="n"/>
+      <c r="AB22" s="14">
+        <f>IF(AA22="","",AA22+5)</f>
+        <v/>
+      </c>
+      <c r="AC22" s="13" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
@@ -9383,10 +10727,20 @@
       <c r="V23" s="9" t="n"/>
       <c r="W23" s="13" t="n"/>
       <c r="X23" s="11">
-        <f>IF(MAX(I23:L23,N23,P23:S23)=0,"",TODAY()-MAX(I23:L23,N23,P23:S23))</f>
+        <f>IF(MAX(I23:L23,N23,P23:S23,AA23,AC23)=0,"",TODAY()-MAX(I23:L23,N23,P23:S23,AA23,AC23))</f>
         <v/>
       </c>
       <c r="Y23" s="9" t="n"/>
+      <c r="Z23" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A23,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A23,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA23" s="13" t="n"/>
+      <c r="AB23" s="14">
+        <f>IF(AA23="","",AA23+5)</f>
+        <v/>
+      </c>
+      <c r="AC23" s="13" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
@@ -9445,10 +10799,20 @@
       <c r="V24" s="9" t="n"/>
       <c r="W24" s="13" t="n"/>
       <c r="X24" s="11">
-        <f>IF(MAX(I24:L24,N24,P24:S24)=0,"",TODAY()-MAX(I24:L24,N24,P24:S24))</f>
+        <f>IF(MAX(I24:L24,N24,P24:S24,AA24,AC24)=0,"",TODAY()-MAX(I24:L24,N24,P24:S24,AA24,AC24))</f>
         <v/>
       </c>
       <c r="Y24" s="9" t="n"/>
+      <c r="Z24" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A24,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A24,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA24" s="13" t="n"/>
+      <c r="AB24" s="14">
+        <f>IF(AA24="","",AA24+5)</f>
+        <v/>
+      </c>
+      <c r="AC24" s="13" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -9507,10 +10871,20 @@
       <c r="V25" s="9" t="n"/>
       <c r="W25" s="13" t="n"/>
       <c r="X25" s="11">
-        <f>IF(MAX(I25:L25,N25,P25:S25)=0,"",TODAY()-MAX(I25:L25,N25,P25:S25))</f>
+        <f>IF(MAX(I25:L25,N25,P25:S25,AA25,AC25)=0,"",TODAY()-MAX(I25:L25,N25,P25:S25,AA25,AC25))</f>
         <v/>
       </c>
       <c r="Y25" s="9" t="n"/>
+      <c r="Z25" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A25,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A25,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA25" s="13" t="n"/>
+      <c r="AB25" s="14">
+        <f>IF(AA25="","",AA25+5)</f>
+        <v/>
+      </c>
+      <c r="AC25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
@@ -9569,10 +10943,20 @@
       <c r="V26" s="9" t="n"/>
       <c r="W26" s="13" t="n"/>
       <c r="X26" s="11">
-        <f>IF(MAX(I26:L26,N26,P26:S26)=0,"",TODAY()-MAX(I26:L26,N26,P26:S26))</f>
+        <f>IF(MAX(I26:L26,N26,P26:S26,AA26,AC26)=0,"",TODAY()-MAX(I26:L26,N26,P26:S26,AA26,AC26))</f>
         <v/>
       </c>
       <c r="Y26" s="9" t="n"/>
+      <c r="Z26" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A26,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A26,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA26" s="13" t="n"/>
+      <c r="AB26" s="14">
+        <f>IF(AA26="","",AA26+5)</f>
+        <v/>
+      </c>
+      <c r="AC26" s="13" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
@@ -9631,10 +11015,20 @@
       <c r="V27" s="9" t="n"/>
       <c r="W27" s="13" t="n"/>
       <c r="X27" s="11">
-        <f>IF(MAX(I27:L27,N27,P27:S27)=0,"",TODAY()-MAX(I27:L27,N27,P27:S27))</f>
+        <f>IF(MAX(I27:L27,N27,P27:S27,AA27,AC27)=0,"",TODAY()-MAX(I27:L27,N27,P27:S27,AA27,AC27))</f>
         <v/>
       </c>
       <c r="Y27" s="9" t="n"/>
+      <c r="Z27" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A27,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A27,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA27" s="13" t="n"/>
+      <c r="AB27" s="14">
+        <f>IF(AA27="","",AA27+5)</f>
+        <v/>
+      </c>
+      <c r="AC27" s="13" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
@@ -9693,10 +11087,20 @@
       <c r="V28" s="9" t="n"/>
       <c r="W28" s="13" t="n"/>
       <c r="X28" s="11">
-        <f>IF(MAX(I28:L28,N28,P28:S28)=0,"",TODAY()-MAX(I28:L28,N28,P28:S28))</f>
+        <f>IF(MAX(I28:L28,N28,P28:S28,AA28,AC28)=0,"",TODAY()-MAX(I28:L28,N28,P28:S28,AA28,AC28))</f>
         <v/>
       </c>
       <c r="Y28" s="9" t="n"/>
+      <c r="Z28" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A28,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A28,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA28" s="13" t="n"/>
+      <c r="AB28" s="14">
+        <f>IF(AA28="","",AA28+5)</f>
+        <v/>
+      </c>
+      <c r="AC28" s="13" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
@@ -9755,10 +11159,20 @@
       <c r="V29" s="9" t="n"/>
       <c r="W29" s="13" t="n"/>
       <c r="X29" s="11">
-        <f>IF(MAX(I29:L29,N29,P29:S29)=0,"",TODAY()-MAX(I29:L29,N29,P29:S29))</f>
+        <f>IF(MAX(I29:L29,N29,P29:S29,AA29,AC29)=0,"",TODAY()-MAX(I29:L29,N29,P29:S29,AA29,AC29))</f>
         <v/>
       </c>
       <c r="Y29" s="9" t="n"/>
+      <c r="Z29" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A29,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A29,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA29" s="13" t="n"/>
+      <c r="AB29" s="14">
+        <f>IF(AA29="","",AA29+5)</f>
+        <v/>
+      </c>
+      <c r="AC29" s="13" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
@@ -9817,10 +11231,20 @@
       <c r="V30" s="9" t="n"/>
       <c r="W30" s="13" t="n"/>
       <c r="X30" s="11">
-        <f>IF(MAX(I30:L30,N30,P30:S30)=0,"",TODAY()-MAX(I30:L30,N30,P30:S30))</f>
+        <f>IF(MAX(I30:L30,N30,P30:S30,AA30,AC30)=0,"",TODAY()-MAX(I30:L30,N30,P30:S30,AA30,AC30))</f>
         <v/>
       </c>
       <c r="Y30" s="9" t="n"/>
+      <c r="Z30" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A30,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A30,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA30" s="13" t="n"/>
+      <c r="AB30" s="14">
+        <f>IF(AA30="","",AA30+5)</f>
+        <v/>
+      </c>
+      <c r="AC30" s="13" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
@@ -9879,10 +11303,20 @@
       <c r="V31" s="9" t="n"/>
       <c r="W31" s="13" t="n"/>
       <c r="X31" s="11">
-        <f>IF(MAX(I31:L31,N31,P31:S31)=0,"",TODAY()-MAX(I31:L31,N31,P31:S31))</f>
+        <f>IF(MAX(I31:L31,N31,P31:S31,AA31,AC31)=0,"",TODAY()-MAX(I31:L31,N31,P31:S31,AA31,AC31))</f>
         <v/>
       </c>
       <c r="Y31" s="9" t="n"/>
+      <c r="Z31" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A31,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A31,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA31" s="13" t="n"/>
+      <c r="AB31" s="14">
+        <f>IF(AA31="","",AA31+5)</f>
+        <v/>
+      </c>
+      <c r="AC31" s="13" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
@@ -9941,10 +11375,20 @@
       <c r="V32" s="9" t="n"/>
       <c r="W32" s="13" t="n"/>
       <c r="X32" s="11">
-        <f>IF(MAX(I32:L32,N32,P32:S32)=0,"",TODAY()-MAX(I32:L32,N32,P32:S32))</f>
+        <f>IF(MAX(I32:L32,N32,P32:S32,AA32,AC32)=0,"",TODAY()-MAX(I32:L32,N32,P32:S32,AA32,AC32))</f>
         <v/>
       </c>
       <c r="Y32" s="9" t="n"/>
+      <c r="Z32" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A32,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A32,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA32" s="13" t="n"/>
+      <c r="AB32" s="14">
+        <f>IF(AA32="","",AA32+5)</f>
+        <v/>
+      </c>
+      <c r="AC32" s="13" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
@@ -10003,10 +11447,20 @@
       <c r="V33" s="9" t="n"/>
       <c r="W33" s="13" t="n"/>
       <c r="X33" s="11">
-        <f>IF(MAX(I33:L33,N33,P33:S33)=0,"",TODAY()-MAX(I33:L33,N33,P33:S33))</f>
+        <f>IF(MAX(I33:L33,N33,P33:S33,AA33,AC33)=0,"",TODAY()-MAX(I33:L33,N33,P33:S33,AA33,AC33))</f>
         <v/>
       </c>
       <c r="Y33" s="9" t="n"/>
+      <c r="Z33" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A33,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A33,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA33" s="13" t="n"/>
+      <c r="AB33" s="14">
+        <f>IF(AA33="","",AA33+5)</f>
+        <v/>
+      </c>
+      <c r="AC33" s="13" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
@@ -10065,10 +11519,20 @@
       <c r="V34" s="9" t="n"/>
       <c r="W34" s="13" t="n"/>
       <c r="X34" s="11">
-        <f>IF(MAX(I34:L34,N34,P34:S34)=0,"",TODAY()-MAX(I34:L34,N34,P34:S34))</f>
+        <f>IF(MAX(I34:L34,N34,P34:S34,AA34,AC34)=0,"",TODAY()-MAX(I34:L34,N34,P34:S34,AA34,AC34))</f>
         <v/>
       </c>
       <c r="Y34" s="9" t="n"/>
+      <c r="Z34" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A34,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A34,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA34" s="13" t="n"/>
+      <c r="AB34" s="14">
+        <f>IF(AA34="","",AA34+5)</f>
+        <v/>
+      </c>
+      <c r="AC34" s="13" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
@@ -10127,10 +11591,20 @@
       <c r="V35" s="9" t="n"/>
       <c r="W35" s="13" t="n"/>
       <c r="X35" s="11">
-        <f>IF(MAX(I35:L35,N35,P35:S35)=0,"",TODAY()-MAX(I35:L35,N35,P35:S35))</f>
+        <f>IF(MAX(I35:L35,N35,P35:S35,AA35,AC35)=0,"",TODAY()-MAX(I35:L35,N35,P35:S35,AA35,AC35))</f>
         <v/>
       </c>
       <c r="Y35" s="9" t="n"/>
+      <c r="Z35" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A35,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A35,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA35" s="13" t="n"/>
+      <c r="AB35" s="14">
+        <f>IF(AA35="","",AA35+5)</f>
+        <v/>
+      </c>
+      <c r="AC35" s="13" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
@@ -10189,10 +11663,20 @@
       <c r="V36" s="9" t="n"/>
       <c r="W36" s="13" t="n"/>
       <c r="X36" s="11">
-        <f>IF(MAX(I36:L36,N36,P36:S36)=0,"",TODAY()-MAX(I36:L36,N36,P36:S36))</f>
+        <f>IF(MAX(I36:L36,N36,P36:S36,AA36,AC36)=0,"",TODAY()-MAX(I36:L36,N36,P36:S36,AA36,AC36))</f>
         <v/>
       </c>
       <c r="Y36" s="9" t="n"/>
+      <c r="Z36" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A36,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A36,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA36" s="13" t="n"/>
+      <c r="AB36" s="14">
+        <f>IF(AA36="","",AA36+5)</f>
+        <v/>
+      </c>
+      <c r="AC36" s="13" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
@@ -10251,10 +11735,20 @@
       <c r="V37" s="9" t="n"/>
       <c r="W37" s="13" t="n"/>
       <c r="X37" s="11">
-        <f>IF(MAX(I37:L37,N37,P37:S37)=0,"",TODAY()-MAX(I37:L37,N37,P37:S37))</f>
+        <f>IF(MAX(I37:L37,N37,P37:S37,AA37,AC37)=0,"",TODAY()-MAX(I37:L37,N37,P37:S37,AA37,AC37))</f>
         <v/>
       </c>
       <c r="Y37" s="9" t="n"/>
+      <c r="Z37" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A37,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A37,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA37" s="13" t="n"/>
+      <c r="AB37" s="14">
+        <f>IF(AA37="","",AA37+5)</f>
+        <v/>
+      </c>
+      <c r="AC37" s="13" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
@@ -10313,10 +11807,20 @@
       <c r="V38" s="9" t="n"/>
       <c r="W38" s="13" t="n"/>
       <c r="X38" s="11">
-        <f>IF(MAX(I38:L38,N38,P38:S38)=0,"",TODAY()-MAX(I38:L38,N38,P38:S38))</f>
+        <f>IF(MAX(I38:L38,N38,P38:S38,AA38,AC38)=0,"",TODAY()-MAX(I38:L38,N38,P38:S38,AA38,AC38))</f>
         <v/>
       </c>
       <c r="Y38" s="9" t="n"/>
+      <c r="Z38" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A38,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A38,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA38" s="13" t="n"/>
+      <c r="AB38" s="14">
+        <f>IF(AA38="","",AA38+5)</f>
+        <v/>
+      </c>
+      <c r="AC38" s="13" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
@@ -10375,10 +11879,20 @@
       <c r="V39" s="9" t="n"/>
       <c r="W39" s="13" t="n"/>
       <c r="X39" s="11">
-        <f>IF(MAX(I39:L39,N39,P39:S39)=0,"",TODAY()-MAX(I39:L39,N39,P39:S39))</f>
+        <f>IF(MAX(I39:L39,N39,P39:S39,AA39,AC39)=0,"",TODAY()-MAX(I39:L39,N39,P39:S39,AA39,AC39))</f>
         <v/>
       </c>
       <c r="Y39" s="9" t="n"/>
+      <c r="Z39" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A39,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A39,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA39" s="13" t="n"/>
+      <c r="AB39" s="14">
+        <f>IF(AA39="","",AA39+5)</f>
+        <v/>
+      </c>
+      <c r="AC39" s="13" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
@@ -10437,10 +11951,20 @@
       <c r="V40" s="9" t="n"/>
       <c r="W40" s="13" t="n"/>
       <c r="X40" s="11">
-        <f>IF(MAX(I40:L40,N40,P40:S40)=0,"",TODAY()-MAX(I40:L40,N40,P40:S40))</f>
+        <f>IF(MAX(I40:L40,N40,P40:S40,AA40,AC40)=0,"",TODAY()-MAX(I40:L40,N40,P40:S40,AA40,AC40))</f>
         <v/>
       </c>
       <c r="Y40" s="9" t="n"/>
+      <c r="Z40" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A40,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A40,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA40" s="13" t="n"/>
+      <c r="AB40" s="14">
+        <f>IF(AA40="","",AA40+5)</f>
+        <v/>
+      </c>
+      <c r="AC40" s="13" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="11" t="inlineStr">
@@ -10499,10 +12023,20 @@
       <c r="V41" s="9" t="n"/>
       <c r="W41" s="13" t="n"/>
       <c r="X41" s="11">
-        <f>IF(MAX(I41:L41,N41,P41:S41)=0,"",TODAY()-MAX(I41:L41,N41,P41:S41))</f>
+        <f>IF(MAX(I41:L41,N41,P41:S41,AA41,AC41)=0,"",TODAY()-MAX(I41:L41,N41,P41:S41,AA41,AC41))</f>
         <v/>
       </c>
       <c r="Y41" s="9" t="n"/>
+      <c r="Z41" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A41,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A41,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA41" s="13" t="n"/>
+      <c r="AB41" s="14">
+        <f>IF(AA41="","",AA41+5)</f>
+        <v/>
+      </c>
+      <c r="AC41" s="13" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
@@ -10561,10 +12095,20 @@
       <c r="V42" s="9" t="n"/>
       <c r="W42" s="13" t="n"/>
       <c r="X42" s="11">
-        <f>IF(MAX(I42:L42,N42,P42:S42)=0,"",TODAY()-MAX(I42:L42,N42,P42:S42))</f>
+        <f>IF(MAX(I42:L42,N42,P42:S42,AA42,AC42)=0,"",TODAY()-MAX(I42:L42,N42,P42:S42,AA42,AC42))</f>
         <v/>
       </c>
       <c r="Y42" s="9" t="n"/>
+      <c r="Z42" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A42,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A42,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA42" s="13" t="n"/>
+      <c r="AB42" s="14">
+        <f>IF(AA42="","",AA42+5)</f>
+        <v/>
+      </c>
+      <c r="AC42" s="13" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
@@ -10623,10 +12167,20 @@
       <c r="V43" s="9" t="n"/>
       <c r="W43" s="13" t="n"/>
       <c r="X43" s="11">
-        <f>IF(MAX(I43:L43,N43,P43:S43)=0,"",TODAY()-MAX(I43:L43,N43,P43:S43))</f>
+        <f>IF(MAX(I43:L43,N43,P43:S43,AA43,AC43)=0,"",TODAY()-MAX(I43:L43,N43,P43:S43,AA43,AC43))</f>
         <v/>
       </c>
       <c r="Y43" s="9" t="n"/>
+      <c r="Z43" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A43,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A43,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA43" s="13" t="n"/>
+      <c r="AB43" s="14">
+        <f>IF(AA43="","",AA43+5)</f>
+        <v/>
+      </c>
+      <c r="AC43" s="13" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
@@ -10685,10 +12239,20 @@
       <c r="V44" s="9" t="n"/>
       <c r="W44" s="13" t="n"/>
       <c r="X44" s="11">
-        <f>IF(MAX(I44:L44,N44,P44:S44)=0,"",TODAY()-MAX(I44:L44,N44,P44:S44))</f>
+        <f>IF(MAX(I44:L44,N44,P44:S44,AA44,AC44)=0,"",TODAY()-MAX(I44:L44,N44,P44:S44,AA44,AC44))</f>
         <v/>
       </c>
       <c r="Y44" s="9" t="n"/>
+      <c r="Z44" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A44,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A44,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA44" s="13" t="n"/>
+      <c r="AB44" s="14">
+        <f>IF(AA44="","",AA44+5)</f>
+        <v/>
+      </c>
+      <c r="AC44" s="13" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
@@ -10747,10 +12311,20 @@
       <c r="V45" s="9" t="n"/>
       <c r="W45" s="13" t="n"/>
       <c r="X45" s="11">
-        <f>IF(MAX(I45:L45,N45,P45:S45)=0,"",TODAY()-MAX(I45:L45,N45,P45:S45))</f>
+        <f>IF(MAX(I45:L45,N45,P45:S45,AA45,AC45)=0,"",TODAY()-MAX(I45:L45,N45,P45:S45,AA45,AC45))</f>
         <v/>
       </c>
       <c r="Y45" s="9" t="n"/>
+      <c r="Z45" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A45,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A45,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA45" s="13" t="n"/>
+      <c r="AB45" s="14">
+        <f>IF(AA45="","",AA45+5)</f>
+        <v/>
+      </c>
+      <c r="AC45" s="13" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
@@ -10809,10 +12383,20 @@
       <c r="V46" s="9" t="n"/>
       <c r="W46" s="13" t="n"/>
       <c r="X46" s="11">
-        <f>IF(MAX(I46:L46,N46,P46:S46)=0,"",TODAY()-MAX(I46:L46,N46,P46:S46))</f>
+        <f>IF(MAX(I46:L46,N46,P46:S46,AA46,AC46)=0,"",TODAY()-MAX(I46:L46,N46,P46:S46,AA46,AC46))</f>
         <v/>
       </c>
       <c r="Y46" s="9" t="n"/>
+      <c r="Z46" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A46,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A46,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA46" s="13" t="n"/>
+      <c r="AB46" s="14">
+        <f>IF(AA46="","",AA46+5)</f>
+        <v/>
+      </c>
+      <c r="AC46" s="13" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
@@ -10871,10 +12455,20 @@
       <c r="V47" s="9" t="n"/>
       <c r="W47" s="13" t="n"/>
       <c r="X47" s="11">
-        <f>IF(MAX(I47:L47,N47,P47:S47)=0,"",TODAY()-MAX(I47:L47,N47,P47:S47))</f>
+        <f>IF(MAX(I47:L47,N47,P47:S47,AA47,AC47)=0,"",TODAY()-MAX(I47:L47,N47,P47:S47,AA47,AC47))</f>
         <v/>
       </c>
       <c r="Y47" s="9" t="n"/>
+      <c r="Z47" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A47,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A47,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA47" s="13" t="n"/>
+      <c r="AB47" s="14">
+        <f>IF(AA47="","",AA47+5)</f>
+        <v/>
+      </c>
+      <c r="AC47" s="13" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
@@ -10933,10 +12527,20 @@
       <c r="V48" s="9" t="n"/>
       <c r="W48" s="13" t="n"/>
       <c r="X48" s="11">
-        <f>IF(MAX(I48:L48,N48,P48:S48)=0,"",TODAY()-MAX(I48:L48,N48,P48:S48))</f>
+        <f>IF(MAX(I48:L48,N48,P48:S48,AA48,AC48)=0,"",TODAY()-MAX(I48:L48,N48,P48:S48,AA48,AC48))</f>
         <v/>
       </c>
       <c r="Y48" s="9" t="n"/>
+      <c r="Z48" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A48,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A48,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA48" s="13" t="n"/>
+      <c r="AB48" s="14">
+        <f>IF(AA48="","",AA48+5)</f>
+        <v/>
+      </c>
+      <c r="AC48" s="13" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
@@ -10995,10 +12599,20 @@
       <c r="V49" s="9" t="n"/>
       <c r="W49" s="13" t="n"/>
       <c r="X49" s="11">
-        <f>IF(MAX(I49:L49,N49,P49:S49)=0,"",TODAY()-MAX(I49:L49,N49,P49:S49))</f>
+        <f>IF(MAX(I49:L49,N49,P49:S49,AA49,AC49)=0,"",TODAY()-MAX(I49:L49,N49,P49:S49,AA49,AC49))</f>
         <v/>
       </c>
       <c r="Y49" s="9" t="n"/>
+      <c r="Z49" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A49,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A49,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA49" s="13" t="n"/>
+      <c r="AB49" s="14">
+        <f>IF(AA49="","",AA49+5)</f>
+        <v/>
+      </c>
+      <c r="AC49" s="13" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
@@ -11057,10 +12671,20 @@
       <c r="V50" s="9" t="n"/>
       <c r="W50" s="13" t="n"/>
       <c r="X50" s="11">
-        <f>IF(MAX(I50:L50,N50,P50:S50)=0,"",TODAY()-MAX(I50:L50,N50,P50:S50))</f>
+        <f>IF(MAX(I50:L50,N50,P50:S50,AA50,AC50)=0,"",TODAY()-MAX(I50:L50,N50,P50:S50,AA50,AC50))</f>
         <v/>
       </c>
       <c r="Y50" s="9" t="n"/>
+      <c r="Z50" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A50,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A50,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA50" s="13" t="n"/>
+      <c r="AB50" s="14">
+        <f>IF(AA50="","",AA50+5)</f>
+        <v/>
+      </c>
+      <c r="AC50" s="13" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
@@ -11119,10 +12743,20 @@
       <c r="V51" s="9" t="n"/>
       <c r="W51" s="13" t="n"/>
       <c r="X51" s="11">
-        <f>IF(MAX(I51:L51,N51,P51:S51)=0,"",TODAY()-MAX(I51:L51,N51,P51:S51))</f>
+        <f>IF(MAX(I51:L51,N51,P51:S51,AA51,AC51)=0,"",TODAY()-MAX(I51:L51,N51,P51:S51,AA51,AC51))</f>
         <v/>
       </c>
       <c r="Y51" s="9" t="n"/>
+      <c r="Z51" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A51,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A51,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA51" s="13" t="n"/>
+      <c r="AB51" s="14">
+        <f>IF(AA51="","",AA51+5)</f>
+        <v/>
+      </c>
+      <c r="AC51" s="13" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
@@ -11181,10 +12815,20 @@
       <c r="V52" s="9" t="n"/>
       <c r="W52" s="13" t="n"/>
       <c r="X52" s="11">
-        <f>IF(MAX(I52:L52,N52,P52:S52)=0,"",TODAY()-MAX(I52:L52,N52,P52:S52))</f>
+        <f>IF(MAX(I52:L52,N52,P52:S52,AA52,AC52)=0,"",TODAY()-MAX(I52:L52,N52,P52:S52,AA52,AC52))</f>
         <v/>
       </c>
       <c r="Y52" s="9" t="n"/>
+      <c r="Z52" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A52,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A52,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA52" s="13" t="n"/>
+      <c r="AB52" s="14">
+        <f>IF(AA52="","",AA52+5)</f>
+        <v/>
+      </c>
+      <c r="AC52" s="13" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
@@ -11243,10 +12887,20 @@
       <c r="V53" s="9" t="n"/>
       <c r="W53" s="13" t="n"/>
       <c r="X53" s="11">
-        <f>IF(MAX(I53:L53,N53,P53:S53)=0,"",TODAY()-MAX(I53:L53,N53,P53:S53))</f>
+        <f>IF(MAX(I53:L53,N53,P53:S53,AA53,AC53)=0,"",TODAY()-MAX(I53:L53,N53,P53:S53,AA53,AC53))</f>
         <v/>
       </c>
       <c r="Y53" s="9" t="n"/>
+      <c r="Z53" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A53,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A53,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA53" s="13" t="n"/>
+      <c r="AB53" s="14">
+        <f>IF(AA53="","",AA53+5)</f>
+        <v/>
+      </c>
+      <c r="AC53" s="13" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
@@ -11305,10 +12959,20 @@
       <c r="V54" s="9" t="n"/>
       <c r="W54" s="13" t="n"/>
       <c r="X54" s="11">
-        <f>IF(MAX(I54:L54,N54,P54:S54)=0,"",TODAY()-MAX(I54:L54,N54,P54:S54))</f>
+        <f>IF(MAX(I54:L54,N54,P54:S54,AA54,AC54)=0,"",TODAY()-MAX(I54:L54,N54,P54:S54,AA54,AC54))</f>
         <v/>
       </c>
       <c r="Y54" s="9" t="n"/>
+      <c r="Z54" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A54,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A54,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA54" s="13" t="n"/>
+      <c r="AB54" s="14">
+        <f>IF(AA54="","",AA54+5)</f>
+        <v/>
+      </c>
+      <c r="AC54" s="13" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
@@ -11367,10 +13031,20 @@
       <c r="V55" s="9" t="n"/>
       <c r="W55" s="13" t="n"/>
       <c r="X55" s="11">
-        <f>IF(MAX(I55:L55,N55,P55:S55)=0,"",TODAY()-MAX(I55:L55,N55,P55:S55))</f>
+        <f>IF(MAX(I55:L55,N55,P55:S55,AA55,AC55)=0,"",TODAY()-MAX(I55:L55,N55,P55:S55,AA55,AC55))</f>
         <v/>
       </c>
       <c r="Y55" s="9" t="n"/>
+      <c r="Z55" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A55,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A55,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA55" s="13" t="n"/>
+      <c r="AB55" s="14">
+        <f>IF(AA55="","",AA55+5)</f>
+        <v/>
+      </c>
+      <c r="AC55" s="13" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
@@ -11429,10 +13103,20 @@
       <c r="V56" s="9" t="n"/>
       <c r="W56" s="13" t="n"/>
       <c r="X56" s="11">
-        <f>IF(MAX(I56:L56,N56,P56:S56)=0,"",TODAY()-MAX(I56:L56,N56,P56:S56))</f>
+        <f>IF(MAX(I56:L56,N56,P56:S56,AA56,AC56)=0,"",TODAY()-MAX(I56:L56,N56,P56:S56,AA56,AC56))</f>
         <v/>
       </c>
       <c r="Y56" s="9" t="n"/>
+      <c r="Z56" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A56,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A56,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA56" s="13" t="n"/>
+      <c r="AB56" s="14">
+        <f>IF(AA56="","",AA56+5)</f>
+        <v/>
+      </c>
+      <c r="AC56" s="13" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
@@ -11491,10 +13175,20 @@
       <c r="V57" s="9" t="n"/>
       <c r="W57" s="13" t="n"/>
       <c r="X57" s="11">
-        <f>IF(MAX(I57:L57,N57,P57:S57)=0,"",TODAY()-MAX(I57:L57,N57,P57:S57))</f>
+        <f>IF(MAX(I57:L57,N57,P57:S57,AA57,AC57)=0,"",TODAY()-MAX(I57:L57,N57,P57:S57,AA57,AC57))</f>
         <v/>
       </c>
       <c r="Y57" s="9" t="n"/>
+      <c r="Z57" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A57,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A57,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA57" s="13" t="n"/>
+      <c r="AB57" s="14">
+        <f>IF(AA57="","",AA57+5)</f>
+        <v/>
+      </c>
+      <c r="AC57" s="13" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
@@ -11553,10 +13247,20 @@
       <c r="V58" s="9" t="n"/>
       <c r="W58" s="13" t="n"/>
       <c r="X58" s="11">
-        <f>IF(MAX(I58:L58,N58,P58:S58)=0,"",TODAY()-MAX(I58:L58,N58,P58:S58))</f>
+        <f>IF(MAX(I58:L58,N58,P58:S58,AA58,AC58)=0,"",TODAY()-MAX(I58:L58,N58,P58:S58,AA58,AC58))</f>
         <v/>
       </c>
       <c r="Y58" s="9" t="n"/>
+      <c r="Z58" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A58,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A58,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA58" s="13" t="n"/>
+      <c r="AB58" s="14">
+        <f>IF(AA58="","",AA58+5)</f>
+        <v/>
+      </c>
+      <c r="AC58" s="13" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="inlineStr">
@@ -11615,10 +13319,20 @@
       <c r="V59" s="9" t="n"/>
       <c r="W59" s="13" t="n"/>
       <c r="X59" s="11">
-        <f>IF(MAX(I59:L59,N59,P59:S59)=0,"",TODAY()-MAX(I59:L59,N59,P59:S59))</f>
+        <f>IF(MAX(I59:L59,N59,P59:S59,AA59,AC59)=0,"",TODAY()-MAX(I59:L59,N59,P59:S59,AA59,AC59))</f>
         <v/>
       </c>
       <c r="Y59" s="9" t="n"/>
+      <c r="Z59" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A59,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A59,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA59" s="13" t="n"/>
+      <c r="AB59" s="14">
+        <f>IF(AA59="","",AA59+5)</f>
+        <v/>
+      </c>
+      <c r="AC59" s="13" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
@@ -11677,10 +13391,20 @@
       <c r="V60" s="9" t="n"/>
       <c r="W60" s="13" t="n"/>
       <c r="X60" s="11">
-        <f>IF(MAX(I60:L60,N60,P60:S60)=0,"",TODAY()-MAX(I60:L60,N60,P60:S60))</f>
+        <f>IF(MAX(I60:L60,N60,P60:S60,AA60,AC60)=0,"",TODAY()-MAX(I60:L60,N60,P60:S60,AA60,AC60))</f>
         <v/>
       </c>
       <c r="Y60" s="9" t="n"/>
+      <c r="Z60" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A60,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A60,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA60" s="13" t="n"/>
+      <c r="AB60" s="14">
+        <f>IF(AA60="","",AA60+5)</f>
+        <v/>
+      </c>
+      <c r="AC60" s="13" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
@@ -11739,25 +13463,40 @@
       <c r="V61" s="9" t="n"/>
       <c r="W61" s="13" t="n"/>
       <c r="X61" s="11">
-        <f>IF(MAX(I61:L61,N61,P61:S61)=0,"",TODAY()-MAX(I61:L61,N61,P61:S61))</f>
+        <f>IF(MAX(I61:L61,N61,P61:S61,AA61,AC61)=0,"",TODAY()-MAX(I61:L61,N61,P61:S61,AA61,AC61))</f>
         <v/>
       </c>
       <c r="Y61" s="9" t="n"/>
+      <c r="Z61" s="11">
+        <f>IFERROR(IF(INDEX(Leads!$X:$X,MATCH($A61,Leads!$A:$A,0))="","",INDEX(Leads!$X:$X,MATCH($A61,Leads!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="AA61" s="13" t="n"/>
+      <c r="AB61" s="14">
+        <f>IF(AA61="","",AA61+5)</f>
+        <v/>
+      </c>
+      <c r="AC61" s="13" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y61"/>
+  <autoFilter ref="A1:AC61"/>
   <conditionalFormatting sqref="M2:M261">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(M2&lt;&gt;"",N2="",M2&lt;TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AB2:AB261">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>AND(AB2&lt;&gt;"",AC2="",AB2&lt;TODAY())</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="O2:O261">
-    <cfRule type="expression" priority="2" dxfId="0">
+    <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(O2&lt;&gt;"",P2="",O2&lt;TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H261">
-    <cfRule type="expression" priority="3" dxfId="1">
+    <cfRule type="expression" priority="4" dxfId="1">
       <formula>OR(H2="Call booked",H2="Call held",H2="Won")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11771,7 +13510,7 @@
     <dataValidation sqref="T2:T261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$C$2:$C$3</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I261 J2:J261 K2:K261 L2:L261 N2:N261 P2:P261 Q2:Q261 R2:R261 S2:S261 W2:W261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Date" error="Enter a date like 2026-09-29" type="date" operator="greaterThan">
+    <dataValidation sqref="I2:I261 J2:J261 K2:K261 L2:L261 N2:N261 P2:P261 Q2:Q261 R2:R261 S2:S261 W2:W261 AA2:AA261 AC2:AC261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Date" error="Enter a date like 2026-09-29" type="date" operator="greaterThan">
       <formula1>45000</formula1>
     </dataValidation>
   </dataValidations>
@@ -12749,7 +14488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12841,16 +14580,28 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Email (second channel)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>If the connection isn't accepted within 5 days, or there's no reply after the first DM, send the cold email from the Leads tab to their verified work email. One email follow-up 5 days later (reply on the same thread): "Bumping this in case it got buried, [Name]. Happy to send the 3-point teardown instead of a call if that's easier."</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Follow-up 1</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>No worries if this is a busy stretch, [Name].
 I put together 3 quick notes on your profile.
@@ -12859,13 +14610,13 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Follow-up 2</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Last one from me, [Name].
 If LinkedIn moves up the list after the raise settles, I'm around.
@@ -12873,53 +14624,53 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Send times</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>India 9 to 11am IST. UK 8 to 10am UK time. Canada and US East 8 to 10am ET. US West 8 to 10am PT. Tuesday to Thursday.</t>
-        </is>
-      </c>
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Limits</t>
+          <t>Send times</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Keep connection requests around 15 to 25 a day. Send by hand, no automation.</t>
+          <t>India 9 to 11am IST. UK 8 to 10am UK time. Canada and US East 8 to 10am ET. US West 8 to 10am PT. Tuesday to Thursday.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Before each send</t>
+          <t>Limits</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>30 seconds on their recent activity: still in role, last post date, any agency or ghostwriter already visible. Fill any [bracketed] line yourself after reading the post.</t>
+          <t>Keep connection requests around 15 to 25 a day. Send by hand, no automation.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>Before each send</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>30 seconds on their recent activity: still in role, last post date, any agency or ghostwriter already visible. Fill any [bracketed] line yourself after reading the post.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>Email rules</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Canada: CASL (relevant to role, unsubscribe). UK: PECR and UK GDPR. US: CAN-SPAM. India: DPDP Act.</t>
         </is>

</xml_diff>

<commit_message>
Add verified emails for 27 leads (Prospeo) and profile corrections
- batches/contacts.csv: lookup results so far (50 of 60 checked)
- Workbook Leads tab: email address, email status and lookup note
- Batch 02: confirmed profiles for Abhishek Murarka and Avni Jain, role and city fixes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCxqvUeG6omvZWYGiRrK1m
</commit_message>
<xml_diff>
--- a/Gliped_Outreach_Tracker.xlsx
+++ b/Gliped_Outreach_Tracker.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Lists" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Leads'!$A$1:$Z$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Leads'!$A$1:$AB$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tracker'!$A$1:$AC$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -800,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z61"/>
+  <dimension ref="A1:AB61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -829,6 +829,8 @@
     <col width="26" customWidth="1" min="24" max="24"/>
     <col width="26" customWidth="1" min="25" max="25"/>
     <col width="60" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="36" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -962,6 +964,16 @@
           <t>Email body</t>
         </is>
       </c>
+      <c r="AA1" s="6" t="inlineStr">
+        <is>
+          <t>Email status</t>
+        </is>
+      </c>
+      <c r="AB1" s="6" t="inlineStr">
+        <is>
+          <t>Email lookup note</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="96" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -1072,7 +1084,11 @@
           <t>India. Warm, respectful tone. Expect a CoS or comms lead in the decision.</t>
         </is>
       </c>
-      <c r="X2" s="9" t="inlineStr"/>
+      <c r="X2" s="9" t="inlineStr">
+        <is>
+          <t>ravi@nuawoman.com</t>
+        </is>
+      </c>
       <c r="Y2" s="7" t="inlineStr">
         <is>
           <t>Nua after the Series C</t>
@@ -1090,6 +1106,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA2" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB2" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="96" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
@@ -1217,6 +1243,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA3" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB3" s="7" t="inlineStr"/>
     </row>
     <row r="4" ht="96" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -1327,7 +1359,11 @@
           <t>UK. Plain and understated. "Might be useful" over "huge opportunity".</t>
         </is>
       </c>
-      <c r="X4" s="9" t="inlineStr"/>
+      <c r="X4" s="9" t="inlineStr">
+        <is>
+          <t>sadra@ryftpay.com</t>
+        </is>
+      </c>
       <c r="Y4" s="7" t="inlineStr">
         <is>
           <t>Ryft's European push</t>
@@ -1345,6 +1381,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA4" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB4" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="96" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -1473,6 +1519,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA5" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="96" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -1601,6 +1653,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA6" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="96" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -1711,7 +1769,11 @@
           <t>SF and Bengaluru. Use a US-direct tone and offer IST or PT slots.</t>
         </is>
       </c>
-      <c r="X7" s="9" t="inlineStr"/>
+      <c r="X7" s="9" t="inlineStr">
+        <is>
+          <t>shourya@flamapp.com</t>
+        </is>
+      </c>
       <c r="Y7" s="7" t="inlineStr">
         <is>
           <t>Flam and US CMOs</t>
@@ -1729,6 +1791,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA7" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB7" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo BOUNCEBAN</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="96" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1839,7 +1911,11 @@
           <t>same company as lead 19. Message Jagnoor first. Don't contact Shashank in the same week. If Jagnoor replies, the pitch can grow into a leadership pair (founder plus CEO). Contact before Shashank ND</t>
         </is>
       </c>
-      <c r="X8" s="9" t="inlineStr"/>
+      <c r="X8" s="9" t="inlineStr">
+        <is>
+          <t>jagnoor.singh@practo.com</t>
+        </is>
+      </c>
       <c r="Y8" s="7" t="inlineStr">
         <is>
           <t>Your first 100 days</t>
@@ -1857,6 +1933,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA8" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB8" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo BOUNCEBAN Prospeo profile linkedin.com/in/jagnoor-singh-65580910 (title still COO)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="96" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
@@ -1985,6 +2071,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA9" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="96" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -2113,6 +2205,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA10" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="96" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
@@ -2223,7 +2321,11 @@
           <t>UK. Direct and specific. He'll spot generic copy immediately. Check for in-house marketing</t>
         </is>
       </c>
-      <c r="X11" s="9" t="inlineStr"/>
+      <c r="X11" s="9" t="inlineStr">
+        <is>
+          <t>theo.saville@cloudnc.com</t>
+        </is>
+      </c>
       <c r="Y11" s="7" t="inlineStr">
         <is>
           <t>The CloudNC story, restarted</t>
@@ -2241,6 +2343,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA11" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB11" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo BOUNCEBAN</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="96" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -2369,6 +2481,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA12" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="96" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
@@ -2479,7 +2597,11 @@
           <t>Canada, Toronto, with a US and YC audience. Short and direct.</t>
         </is>
       </c>
-      <c r="X13" s="9" t="inlineStr"/>
+      <c r="X13" s="9" t="inlineStr">
+        <is>
+          <t>raghav@withterminal.com</t>
+        </is>
+      </c>
       <c r="Y13" s="7" t="inlineStr">
         <is>
           <t>Hiring after the Series A</t>
@@ -2497,6 +2619,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA13" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB13" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="96" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -2607,7 +2739,11 @@
           <t>Canada, Alberta. Respectful. He likely has advisers, so expect a gatekeeper. Former Alberta minister</t>
         </is>
       </c>
-      <c r="X14" s="9" t="inlineStr"/>
+      <c r="X14" s="9" t="inlineStr">
+        <is>
+          <t>doug.schweitzer@ultimarii.com</t>
+        </is>
+      </c>
       <c r="Y14" s="7" t="inlineStr">
         <is>
           <t>From minister to founder</t>
@@ -2625,6 +2761,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA14" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB14" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo BOUNCEBAN</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="96" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -2735,7 +2881,11 @@
           <t>Quebec. Offer French. Polite and practical. Active last 30 days; offer French</t>
         </is>
       </c>
-      <c r="X15" s="9" t="inlineStr"/>
+      <c r="X15" s="9" t="inlineStr">
+        <is>
+          <t>gabriel@scopia.tech</t>
+        </is>
+      </c>
       <c r="Y15" s="7" t="inlineStr">
         <is>
           <t>Scopia's next chapter</t>
@@ -2753,6 +2903,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA15" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB15" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo BOUNCEBAN</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="96" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -2881,6 +3041,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA16" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB16" s="7" t="inlineStr"/>
     </row>
     <row r="17" ht="96" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
@@ -3009,6 +3175,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA17" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB17" s="7" t="inlineStr"/>
     </row>
     <row r="18" ht="96" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -3137,6 +3309,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA18" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB18" s="7" t="inlineStr"/>
     </row>
     <row r="19" ht="96" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
@@ -3247,7 +3425,11 @@
           <t>US East. Direct.</t>
         </is>
       </c>
-      <c r="X19" s="9" t="inlineStr"/>
+      <c r="X19" s="9" t="inlineStr">
+        <is>
+          <t>shishir@helogen.com</t>
+        </is>
+      </c>
       <c r="Y19" s="7" t="inlineStr">
         <is>
           <t>Explaining Helogen</t>
@@ -3265,6 +3447,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA19" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB19" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP Prospeo profile linkedin.com/in/shishir-b-40ba0a126 (Helogen CEO)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="96" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -3371,7 +3563,11 @@
           <t>only after lead 7 has been contacted and at least a week has passed. The likely route is through his comms or CoS. India, senior. Very respectful and short. Wait 1 week after Jagnoor</t>
         </is>
       </c>
-      <c r="X20" s="9" t="inlineStr"/>
+      <c r="X20" s="9" t="inlineStr">
+        <is>
+          <t>shashank@centai.in</t>
+        </is>
+      </c>
       <c r="Y20" s="7" t="inlineStr">
         <is>
           <t>The chairman's voice</t>
@@ -3389,6 +3585,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA20" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB20" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP Address is at Cent (his preventive-health company) not Practo</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="96" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
@@ -3499,7 +3705,11 @@
           <t>US West. Numbers-first. He'll judge Gliped on its own profile, so make sure it's current. Pitch time and reach not starting</t>
         </is>
       </c>
-      <c r="X21" s="9" t="inlineStr"/>
+      <c r="X21" s="9" t="inlineStr">
+        <is>
+          <t>ilan@sapiom.ai</t>
+        </is>
+      </c>
       <c r="Y21" s="7" t="inlineStr">
         <is>
           <t>Your weekly hours back</t>
@@ -3517,6 +3727,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA21" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB21" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="96" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -3635,7 +3855,11 @@
           <t>Co-founders Ujjwal Sukheja and Saran S. also post. Pitch Aniket first.</t>
         </is>
       </c>
-      <c r="X22" s="9" t="inlineStr"/>
+      <c r="X22" s="9" t="inlineStr">
+        <is>
+          <t>aniket@justswish.in</t>
+        </is>
+      </c>
       <c r="Y22" s="7" t="inlineStr">
         <is>
           <t>Swish's founder story</t>
@@ -3653,6 +3877,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA22" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB22" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="96" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
@@ -3771,7 +4005,11 @@
           <t>Deep tech, government and defence buyers. Keep it formal.</t>
         </is>
       </c>
-      <c r="X23" s="9" t="inlineStr"/>
+      <c r="X23" s="9" t="inlineStr">
+        <is>
+          <t>sunil@qnulabs.com</t>
+        </is>
+      </c>
       <c r="Y23" s="7" t="inlineStr">
         <is>
           <t>Quantum-safe, explained</t>
@@ -3789,6 +4027,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA23" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB23" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="96" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
@@ -3907,7 +4155,11 @@
           <t>Check whether he already posts on YouTube or X. If so, pitch repurposing onto LinkedIn.</t>
         </is>
       </c>
-      <c r="X24" s="9" t="inlineStr"/>
+      <c r="X24" s="9" t="inlineStr">
+        <is>
+          <t>prashant.shah@definedge.com</t>
+        </is>
+      </c>
       <c r="Y24" s="7" t="inlineStr">
         <is>
           <t>Your credentials, visible</t>
@@ -3925,6 +4177,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA24" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB24" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP Prospeo headline: Co-founder &amp; CEO</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="96" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
@@ -4061,6 +4323,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA25" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB25" s="7" t="inlineStr"/>
     </row>
     <row r="26" ht="96" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
@@ -4193,6 +4461,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA26" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB26" s="7" t="inlineStr"/>
     </row>
     <row r="27" ht="96" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
@@ -4303,7 +4577,11 @@
           <t>Confirm profile before sending.</t>
         </is>
       </c>
-      <c r="X27" s="9" t="inlineStr"/>
+      <c r="X27" s="9" t="inlineStr">
+        <is>
+          <t>abhishek@circolife.com</t>
+        </is>
+      </c>
       <c r="Y27" s="7" t="inlineStr">
         <is>
           <t>Cooling as a category</t>
@@ -4321,6 +4599,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA27" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB27" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP PROFILE https://www.linkedin.com/in/abhishek-murarka-633b876 (CEO &amp; Co-Founder Circolife)</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="96" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
@@ -4453,6 +4741,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA28" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB28" s="7" t="inlineStr"/>
     </row>
     <row r="29" ht="96" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
@@ -4585,6 +4879,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA29" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB29" s="7" t="inlineStr"/>
     </row>
     <row r="30" ht="96" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
@@ -4717,6 +5017,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA30" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB30" s="7" t="inlineStr"/>
     </row>
     <row r="31" ht="96" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
@@ -4827,7 +5133,11 @@
           <t>Confirm profile. Pre-seed budget, so offer the pilot.</t>
         </is>
       </c>
-      <c r="X31" s="9" t="inlineStr"/>
+      <c r="X31" s="9" t="inlineStr">
+        <is>
+          <t>avni@nuvah.in</t>
+        </is>
+      </c>
       <c r="Y31" s="7" t="inlineStr">
         <is>
           <t>24 prototypes is content</t>
@@ -4845,6 +5155,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA31" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB31" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP PROFILE https://www.linkedin.com/in/avni-jain-05b45448 (Founder &amp; CEO Nuvah)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="96" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
@@ -4963,7 +5283,11 @@
           <t>Likely has comms support. Ask who owns his LinkedIn.</t>
         </is>
       </c>
-      <c r="X32" s="9" t="inlineStr"/>
+      <c r="X32" s="9" t="inlineStr">
+        <is>
+          <t>charlie@scan.com</t>
+        </is>
+      </c>
       <c r="Y32" s="7" t="inlineStr">
         <is>
           <t>Scan.com's US chapter</t>
@@ -4981,6 +5305,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA32" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB32" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP Based in Atlanta per Prospeo</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="96" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
@@ -5099,7 +5433,11 @@
           <t>The 'resigns' post is an April Fools joke. He's still CEO.</t>
         </is>
       </c>
-      <c r="X33" s="9" t="inlineStr"/>
+      <c r="X33" s="9" t="inlineStr">
+        <is>
+          <t>charlie.cook@rightcharge.co.uk</t>
+        </is>
+      </c>
       <c r="Y33" s="7" t="inlineStr">
         <is>
           <t>Rightcharge across Europe</t>
@@ -5117,6 +5455,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA33" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB33" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="96" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
@@ -5231,7 +5579,11 @@
         </is>
       </c>
       <c r="W34" s="7" t="inlineStr"/>
-      <c r="X34" s="9" t="inlineStr"/>
+      <c r="X34" s="9" t="inlineStr">
+        <is>
+          <t>koji@ki-hydrogen.com</t>
+        </is>
+      </c>
       <c r="Y34" s="7" t="inlineStr">
         <is>
           <t>Making Ki 13 stick</t>
@@ -5249,6 +5601,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA34" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB34" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo BOUNCEBAN Domain is the old Ki Hydrogen name; still verified</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="96" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
@@ -5363,7 +5725,11 @@
         </is>
       </c>
       <c r="W35" s="7" t="inlineStr"/>
-      <c r="X35" s="9" t="inlineStr"/>
+      <c r="X35" s="9" t="inlineStr">
+        <is>
+          <t>francisco@geosurge.ai</t>
+        </is>
+      </c>
       <c r="Y35" s="7" t="inlineStr">
         <is>
           <t>Your own AI visibility</t>
@@ -5381,6 +5747,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA35" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB35" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="96" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
@@ -5517,6 +5893,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA36" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB36" s="7" t="inlineStr"/>
     </row>
     <row r="37" ht="96" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
@@ -5635,7 +6017,11 @@
           <t>Co-founder Max Clarke. Big brand, so expect a comms team.</t>
         </is>
       </c>
-      <c r="X37" s="9" t="inlineStr"/>
+      <c r="X37" s="9" t="inlineStr">
+        <is>
+          <t>lestat@healf.com</t>
+        </is>
+      </c>
       <c r="Y37" s="7" t="inlineStr">
         <is>
           <t>Healf, week by week</t>
@@ -5653,6 +6039,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA37" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB37" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="96" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
@@ -5771,7 +6167,11 @@
           <t>Low fit for ghostwriting. Only pitch strategy.</t>
         </is>
       </c>
-      <c r="X38" s="9" t="inlineStr"/>
+      <c r="X38" s="9" t="inlineStr">
+        <is>
+          <t>jon@marker.page</t>
+        </is>
+      </c>
       <c r="Y38" s="7" t="inlineStr">
         <is>
           <t>Distribution, not writing</t>
@@ -5789,6 +6189,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA38" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB38" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="96" customHeight="1">
       <c r="A39" s="7" t="inlineStr">
@@ -5925,6 +6335,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA39" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB39" s="7" t="inlineStr"/>
     </row>
     <row r="40" ht="96" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
@@ -6053,6 +6469,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA40" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB40" s="7" t="inlineStr"/>
     </row>
     <row r="41" ht="96" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
@@ -6184,6 +6606,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA41" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB41" s="7" t="inlineStr"/>
     </row>
     <row r="42" ht="96" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
@@ -6316,6 +6744,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA42" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB42" s="7" t="inlineStr"/>
     </row>
     <row r="43" ht="96" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
@@ -6434,7 +6868,11 @@
           <t>Writer himself, so pitch strategy over ghostwriting.</t>
         </is>
       </c>
-      <c r="X43" s="9" t="inlineStr"/>
+      <c r="X43" s="9" t="inlineStr">
+        <is>
+          <t>david@onixai.ai</t>
+        </is>
+      </c>
       <c r="Y43" s="7" t="inlineStr">
         <is>
           <t>Onix and your voice</t>
@@ -6452,6 +6890,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA43" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB43" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP Prospeo lists Onix HQ as Montreal (sheet says Ottawa)</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="96" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
@@ -6570,7 +7018,11 @@
           <t>Likely has an in-house comms team. Pitch executive content support.</t>
         </is>
       </c>
-      <c r="X44" s="9" t="inlineStr"/>
+      <c r="X44" s="9" t="inlineStr">
+        <is>
+          <t>kyle.braatz@fullscript.com</t>
+        </is>
+      </c>
       <c r="Y44" s="7" t="inlineStr">
         <is>
           <t>Fullscript's CEO voice</t>
@@ -6588,6 +7040,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA44" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB44" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo BOUNCEBAN</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="96" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
@@ -6724,6 +7186,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA45" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB45" s="7" t="inlineStr"/>
     </row>
     <row r="46" ht="96" customHeight="1">
       <c r="A46" s="7" t="inlineStr">
@@ -6842,7 +7310,11 @@
           <t>Confirm the funding date before sending. Write in French.</t>
         </is>
       </c>
-      <c r="X46" s="9" t="inlineStr"/>
+      <c r="X46" s="9" t="inlineStr">
+        <is>
+          <t>sgarneau@micrologic.ca</t>
+        </is>
+      </c>
       <c r="Y46" s="7" t="inlineStr">
         <is>
           <t>Micrologic et le cloud souverain</t>
@@ -6860,6 +7332,16 @@
 Pas pertinent? Répondez « non » et je ne vous relancerai pas.</t>
         </is>
       </c>
+      <c r="AA46" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB46" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP Prospeo places Micrologic in Québec City (sheet says Montreal)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="96" customHeight="1">
       <c r="A47" s="7" t="inlineStr">
@@ -6996,6 +7478,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA47" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB47" s="7" t="inlineStr"/>
     </row>
     <row r="48" ht="96" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
@@ -7113,7 +7601,11 @@
           <t>Nurture. Trigger is older than 90 days. Revisit on the next trigger.</t>
         </is>
       </c>
-      <c r="X48" s="9" t="inlineStr"/>
+      <c r="X48" s="9" t="inlineStr">
+        <is>
+          <t>kimia@nationgraph.com</t>
+        </is>
+      </c>
       <c r="Y48" s="7" t="inlineStr">
         <is>
           <t>NationGraph, steadily</t>
@@ -7131,6 +7623,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA48" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB48" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="96" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
@@ -7263,6 +7765,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA49" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB49" s="7" t="inlineStr"/>
     </row>
     <row r="50" ht="96" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
@@ -7395,6 +7903,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA50" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AB50" s="7" t="inlineStr"/>
     </row>
     <row r="51" ht="96" customHeight="1">
       <c r="A51" s="7" t="inlineStr">
@@ -7509,7 +8023,11 @@
           <t>Launch, not a funding round. Check whether there was a raise.</t>
         </is>
       </c>
-      <c r="X51" s="9" t="inlineStr"/>
+      <c r="X51" s="9" t="inlineStr">
+        <is>
+          <t>sumit@getmakeos.com</t>
+        </is>
+      </c>
       <c r="Y51" s="7" t="inlineStr">
         <is>
           <t>MakeOS, founder-led</t>
@@ -7527,6 +8045,16 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA51" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="AB51" s="7" t="inlineStr">
+        <is>
+          <t>Prospeo SMTP</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="96" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
@@ -7655,6 +8183,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA52" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="AB52" s="7" t="inlineStr"/>
     </row>
     <row r="53" ht="96" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
@@ -7787,6 +8321,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA53" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="AB53" s="7" t="inlineStr"/>
     </row>
     <row r="54" ht="96" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
@@ -7923,6 +8463,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA54" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="AB54" s="7" t="inlineStr"/>
     </row>
     <row r="55" ht="96" customHeight="1">
       <c r="A55" s="7" t="inlineStr">
@@ -8055,6 +8601,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA55" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="AB55" s="7" t="inlineStr"/>
     </row>
     <row r="56" ht="96" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
@@ -8187,6 +8739,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA56" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="AB56" s="7" t="inlineStr"/>
     </row>
     <row r="57" ht="96" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
@@ -8323,6 +8881,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA57" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="AB57" s="7" t="inlineStr"/>
     </row>
     <row r="58" ht="96" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
@@ -8455,6 +9019,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA58" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="AB58" s="7" t="inlineStr"/>
     </row>
     <row r="59" ht="96" customHeight="1">
       <c r="A59" s="7" t="inlineStr">
@@ -8583,6 +9153,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA59" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="AB59" s="7" t="inlineStr"/>
     </row>
     <row r="60" ht="96" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
@@ -8715,6 +9291,12 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA60" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="AB60" s="7" t="inlineStr"/>
     </row>
     <row r="61" ht="96" customHeight="1">
       <c r="A61" s="7" t="inlineStr">
@@ -8847,16 +9429,30 @@
 Not relevant? Reply "no" and I won't follow up.</t>
         </is>
       </c>
+      <c r="AA61" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="AB61" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z61"/>
+  <autoFilter ref="A1:AB61"/>
   <conditionalFormatting sqref="J2:J261">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AA2:AA261">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Verified"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
+      <formula>"Not found"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="R2:R261">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
       <formula>"Priority"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Add downloadable PDF lead pack (contacts, messages, cold emails)
batches/build_pdf.py renders Gliped_Lead_Pack.pdf from the workbook:
summary, contact list with email status, and one card per lead.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCxqvUeG6omvZWYGiRrK1m
</commit_message>
<xml_diff>
--- a/Gliped_Outreach_Tracker.xlsx
+++ b/Gliped_Outreach_Tracker.xlsx
@@ -4061,7 +4061,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Co-founder</t>
+          <t>Co-founder &amp; CEO</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
@@ -4507,12 +4507,12 @@
       <c r="H27" s="7" t="inlineStr"/>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/people/?keywords=Abhishek%20Murarka%20Circolife</t>
+          <t>https://www.linkedin.com/in/abhishek-murarka-633b876</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -4574,7 +4574,7 @@
       </c>
       <c r="W27" s="7" t="inlineStr">
         <is>
-          <t>Confirm profile before sending.</t>
+          <t>Profile confirmed via Prospeo (CEO &amp; Co-Founder, Circolife). Indexed posts under this name were a different person.</t>
         </is>
       </c>
       <c r="X27" s="9" t="inlineStr">
@@ -5063,12 +5063,12 @@
       <c r="H31" s="7" t="inlineStr"/>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/people/?keywords=Avni%20Jain%20Nuvah</t>
+          <t>https://www.linkedin.com/in/avni-jain-05b45448</t>
         </is>
       </c>
       <c r="J31" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -5130,7 +5130,7 @@
       </c>
       <c r="W31" s="7" t="inlineStr">
         <is>
-          <t>Confirm profile. Pre-seed budget, so offer the pilot.</t>
+          <t>Profile confirmed via Prospeo (Founder &amp; CEO, Nuvah). Pre-seed budget.</t>
         </is>
       </c>
       <c r="X31" s="9" t="inlineStr">
@@ -6789,7 +6789,7 @@
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="I43" s="8" t="inlineStr">
@@ -7231,7 +7231,7 @@
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Québec City</t>
         </is>
       </c>
       <c r="I46" s="8" t="inlineStr">

</xml_diff>